<commit_message>
Update GPS data Excel file
</commit_message>
<xml_diff>
--- a/gps_data.xlsx
+++ b/gps_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,3641 +448,3641 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{A0D18F36-EA14-4F20-8765-A379DCEAA9BB}.jpg</t>
+          <t>{780461B9-3366-430D-BF71-0340723D371F}.jpg</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36.23093380555556</v>
+        <v>36.21637075</v>
       </c>
       <c r="C2" t="n">
-        <v>36.20075208333333</v>
+        <v>36.15504469444444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>{06261D46-239D-4BDA-8AEB-F761F35C0249}.jpg</t>
+          <t>{E52E9E22-3D04-47B6-A1C7-62C91B1A2F2D}.jpg</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37.75729919444444</v>
+        <v>36.56528158333333</v>
       </c>
       <c r="C3" t="n">
-        <v>38.25585708333333</v>
+        <v>36.15630683888889</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{4A5FE300-7542-4021-A196-C09A0E8D542E}.jpg</t>
+          <t>{A0678E82-032A-4D3A-B176-A9FA1FE066D9}.jpg</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37.76518805555556</v>
+        <v>37.76613088888889</v>
       </c>
       <c r="C4" t="n">
-        <v>38.26533038888889</v>
+        <v>38.266975575</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>{F8E6D8C1-7DC7-40D2-9BE2-A7D5F653E380}.jpg</t>
+          <t>{FAEB5345-2C23-4AF0-8A3F-3B5D19D14C64}.jpg</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>36.25972861111111</v>
+        <v>37.55962666666667</v>
       </c>
       <c r="C5" t="n">
-        <v>36.20639278888889</v>
+        <v>36.92028999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{C79931AC-1A1F-4906-8761-5E276EC978EF}.jpg</t>
+          <t>{1A8FF8A6-63FE-4F2F-99FF-CD4B1E3DD047}.jpg</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36.23457488055556</v>
+        <v>36.23682021111111</v>
       </c>
       <c r="C6" t="n">
-        <v>36.16567141666666</v>
+        <v>36.165431</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{2A8304E5-B65C-4A49-A745-FD29854CEC7A}.jpg</t>
+          <t>{6B3B4F05-418D-4318-80A0-67FEEE51669C}.jpg</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37.7519047</v>
+        <v>36.23060205555556</v>
       </c>
       <c r="C7" t="n">
-        <v>38.24508180555556</v>
+        <v>36.19999630555555</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>{C165CBE8-C191-4C8A-AD79-ACB5DC61936C}.jpg</t>
+          <t>{533D50D1-37C8-4C1D-8FBE-6BA7CCA620AF}.jpg</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>37.58274658333334</v>
+        <v>37.57157127222222</v>
       </c>
       <c r="C8" t="n">
-        <v>36.88289466666667</v>
+        <v>36.93660743888888</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>{64168C52-3BE4-43EA-8E3B-0999F05147AC}.jpg</t>
+          <t>{09F10EDC-083A-4F26-BB6C-A9AE0CCD766B}.jpg</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>36.20614769444445</v>
+        <v>37.57178513888889</v>
       </c>
       <c r="C9" t="n">
-        <v>36.15642387777778</v>
+        <v>36.93474944722222</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>{246A5A81-F042-4258-A6C2-A4F061E2D0BB}.jpg</t>
+          <t>{D301AEB0-492E-41E4-8D0C-009DEF9F0382}.jpg</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>36.22787969444445</v>
+        <v>37.57303544444445</v>
       </c>
       <c r="C10" t="n">
-        <v>36.14938769444444</v>
+        <v>36.93914701111111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>{3F02D8E9-773E-47CD-8946-841459249D09}.jpg</t>
+          <t>{F4FC4A8F-455C-4FE4-8EC1-5A90CDA778F0}.jpg</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>36.20548883333333</v>
+        <v>36.20707975000001</v>
       </c>
       <c r="C11" t="n">
-        <v>36.15434047777778</v>
+        <v>36.15848142777778</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>{8677E52A-A4A6-47AE-B373-0A891D0BAE64}.jpg</t>
+          <t>{06261D46-239D-4BDA-8AEB-F761F35C0249}.jpg</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>36.20174878888889</v>
+        <v>37.75729919444444</v>
       </c>
       <c r="C12" t="n">
-        <v>36.16428277777778</v>
+        <v>38.25585708333333</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>{BC1D7E63-7E14-49A5-BDE9-A4FF91774D7D}.jpg</t>
+          <t>{51490BFF-82E7-4BEF-81D5-C1560BD38627}.jpg</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>36.21394394444444</v>
+        <v>37.57397816666667</v>
       </c>
       <c r="C13" t="n">
-        <v>36.16930606111111</v>
+        <v>36.93450889722222</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>{4B067E7F-6299-4C82-A2A3-F9903425355B}.jpg</t>
+          <t>{902AF0E6-0DC8-4F1C-BAD3-A44A382DB66F}.jpg</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>36.20492681111111</v>
+        <v>37.76309269444445</v>
       </c>
       <c r="C14" t="n">
-        <v>36.15883581666667</v>
+        <v>38.2394074</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>{6A6ED554-4709-4BDA-9709-BECEB8F41628}.jpg</t>
+          <t>{BA7A9046-BD7E-4862-850D-A9B2DE988431}.jpg</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37.57207012777778</v>
+        <v>37.574970675</v>
       </c>
       <c r="C15" t="n">
-        <v>36.92389843055555</v>
+        <v>36.93343080499999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>{64F928F8-E576-42EC-B868-2AC2609D1CB5}.jpg</t>
+          <t>{EB274B9F-248D-4EB9-B173-53CC6BC5035C}.jpg</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>37.57297852777778</v>
+        <v>37.77169581388889</v>
       </c>
       <c r="C16" t="n">
-        <v>36.93573819166667</v>
+        <v>38.26375855555555</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>{ACED80DF-AC07-4AC7-A414-60E43822762C}.jpg</t>
+          <t>{93C31A94-5FB3-4199-9685-EECC1833BC93}.jpg</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>37.77459511111111</v>
+        <v>37.76993075277777</v>
       </c>
       <c r="C17" t="n">
-        <v>38.26554547222222</v>
+        <v>38.26451266666667</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>{7131FB9E-B9E7-4612-8926-04EFF43110E2}.jpg</t>
+          <t>{015EA546-5006-4ECD-A229-E87B39B802AA}.jpg</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>37.76333980555555</v>
+        <v>37.77459511111111</v>
       </c>
       <c r="C18" t="n">
-        <v>38.2421846</v>
+        <v>38.26554547222222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>{0A76082E-A7E6-49E8-B505-DF818E9CFFC7}.jpg</t>
+          <t>{EC37422A-5C73-47B5-9212-F7979C986E43}.jpg</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>36.21239963888889</v>
+        <v>36.25974068055555</v>
       </c>
       <c r="C19" t="n">
-        <v>36.14170272222222</v>
+        <v>36.20637169444445</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>{7E41172C-78FD-4402-9ECF-1583F236ACC3}.jpg</t>
+          <t>{6DE016A3-15FD-4DB6-B0FE-40295FFE37D1}.jpg</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>36.21654111111111</v>
+        <v>36.20635880555556</v>
       </c>
       <c r="C20" t="n">
-        <v>36.15421251944444</v>
+        <v>36.15690767222222</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>{9E525EE6-ED31-4103-86E1-0F89C53E89C2}.jpg</t>
+          <t>{E536BE4A-A604-4313-BC64-2876374E677F}.jpg</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>37.76260077777778</v>
+        <v>37.76464019444445</v>
       </c>
       <c r="C21" t="n">
-        <v>38.29404586111111</v>
+        <v>38.27032038055555</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>{9CB58159-DB90-4641-BAAE-DA7D123CF1CA}.jpg</t>
+          <t>{4A5FE300-7542-4021-A196-C09A0E8D542E}.jpg</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>36.21722031305556</v>
+        <v>37.76518805555556</v>
       </c>
       <c r="C22" t="n">
-        <v>36.15681531666667</v>
+        <v>38.26533038888889</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>{4C0E89B0-626A-42D6-BB95-03ABF20E6B8D}.jpg</t>
+          <t>{340592C4-441E-4BB9-AFA9-796650C22585}.jpg</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>36.21713776305555</v>
+        <v>36.20312220277778</v>
       </c>
       <c r="C23" t="n">
-        <v>36.15580826944444</v>
+        <v>36.15145024444444</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>{C40C3F47-F5F4-4194-B2A9-09D274C6650A}.jpg</t>
+          <t>{869B730A-D1B9-4DFB-8841-1DD70CFEBD82}.jpg</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>37.0627124</v>
+        <v>36.21746742222222</v>
       </c>
       <c r="C24" t="n">
-        <v>36.23670659972223</v>
+        <v>36.14187011111111</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>{DBE68764-1740-4D57-894C-0996AF790A55}.jpg</t>
+          <t>{EECF3874-303B-44C7-A044-8C7A2308204B}.jpg</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>36.5663675</v>
+        <v>36.19847755555555</v>
       </c>
       <c r="C25" t="n">
-        <v>36.15448655555556</v>
+        <v>36.15426723055555</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>{E956CAA0-2EDF-4A8F-8FCA-A1EC7F9F80EA}.jpg</t>
+          <t>{7E41172C-78FD-4402-9ECF-1583F236ACC3}.jpg</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>37.57699175</v>
+        <v>36.21654111111111</v>
       </c>
       <c r="C26" t="n">
-        <v>36.91670757722222</v>
+        <v>36.15421251944444</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>{3CEF804A-20EB-4D03-9DFB-B5D29F4A7542}.jpg</t>
+          <t>{21254F46-EE21-4441-984B-01841C143E16}.jpg</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>36.2111895</v>
+        <v>36.2037808</v>
       </c>
       <c r="C27" t="n">
-        <v>36.16153138888889</v>
+        <v>36.160363</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>{EE373BCB-3DB3-49EB-8390-A62561B0A358}.jpg</t>
+          <t>{068E9554-8EFF-4FCE-9CDC-1101FD7FA241}.jpg</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>37.55979833333333</v>
+        <v>36.25975647222222</v>
       </c>
       <c r="C28" t="n">
-        <v>36.91985833333333</v>
+        <v>36.20639878888889</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>{DE6237B2-43FB-407B-8D16-D0280AA530D0}.jpg</t>
+          <t>{975C5CBA-9329-4F97-88D8-4B156D764FF6}.jpg</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>36.23085997222223</v>
+        <v>36.2188823</v>
       </c>
       <c r="C29" t="n">
-        <v>36.19969302777778</v>
+        <v>36.1620305</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>{2C076564-83C0-41A5-AA77-05B8090B1AED}.jpg</t>
+          <t>{B13E60C2-7DF5-47D0-9057-E7AD84699544}.jpg</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>37.74773097222222</v>
+        <v>37.76191227777777</v>
       </c>
       <c r="C30" t="n">
-        <v>38.24966688888889</v>
+        <v>38.29055369444444</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>{6AF44EB2-4F33-44F6-82BD-E746DE95516C}.jpg</t>
+          <t>{81011EC3-C0CB-40B2-8ACB-34FACE9B1E9C}.jpg</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>36.206336575</v>
+        <v>36.2263936</v>
       </c>
       <c r="C31" t="n">
-        <v>36.15693163888889</v>
+        <v>36.1510569</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>{D9FE652D-5354-4AE9-8892-7A7FC3273827}.jpg</t>
+          <t>{4DC84356-E1BD-4BAB-92BE-745F9604D49C}.jpg</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>36.19907777777777</v>
+        <v>37.09941488888889</v>
       </c>
       <c r="C32" t="n">
-        <v>36.15013055555556</v>
+        <v>36.63670741111111</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>{E5D2916C-514A-4A1A-890F-E4A6DEF0F8D1}.jpg</t>
+          <t>{F13B5AD2-FC07-4102-BD96-3484E1E0DEB4}.jpg</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>37.76167088888889</v>
+        <v>37.76299483333333</v>
       </c>
       <c r="C33" t="n">
-        <v>38.26634933333333</v>
+        <v>38.29020973055555</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>{0F27053B-62EE-42CE-AABD-98680EF9C411}.jpg</t>
+          <t>{5A3A809A-E6C7-4A7B-97D2-C071B20C1416}.jpg</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>36.22748977777778</v>
+        <v>37.771418625</v>
       </c>
       <c r="C34" t="n">
-        <v>36.15124046944445</v>
+        <v>38.26922974444444</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>{BA7A9046-BD7E-4862-850D-A9B2DE988431}.jpg</t>
+          <t>{D9FE652D-5354-4AE9-8892-7A7FC3273827}.jpg</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>37.574970675</v>
+        <v>36.19907777777777</v>
       </c>
       <c r="C35" t="n">
-        <v>36.93343080499999</v>
+        <v>36.15013055555556</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>{5BA2AAD0-5AE3-4261-9233-4E241D59B065}.jpg</t>
+          <t>{6D52D63A-D29B-415F-B136-FCFDF6BCFFFF}.jpg</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>36.22861575</v>
+        <v>36.21747463722222</v>
       </c>
       <c r="C36" t="n">
-        <v>36.19683311111111</v>
+        <v>36.16127780555556</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>{08CD4653-870D-4E6A-8D26-CD71C982C3D1}.jpg</t>
+          <t>{D593BFFF-7803-49A3-9973-883F1A3DD122}.jpg</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>36.23115022222223</v>
+        <v>37.7638975</v>
       </c>
       <c r="C37" t="n">
-        <v>36.19971825</v>
+        <v>38.27213311111111</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>{D1AD5CAC-68F7-4447-B32D-4155C22BC087}.jpg</t>
+          <t>{DACF98B6-F238-496B-8AE1-9BD115939851}.jpg</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>37.75662058333333</v>
+        <v>36.21453055555556</v>
       </c>
       <c r="C38" t="n">
-        <v>38.24547044444444</v>
+        <v>36.14272777777778</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>{B72E134E-3779-4EB8-9C30-42E284F8E511}.jpg</t>
+          <t>{0450CBDA-5560-41B1-9C27-00C1B01BC741}.jpg</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>37.57437756666667</v>
+        <v>37.76594458333334</v>
       </c>
       <c r="C39" t="n">
-        <v>36.93379684527778</v>
+        <v>38.26616363888889</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>{136B3821-143F-4048-BF13-D14D0CA38227}.jpg</t>
+          <t>{F9E69747-3A8E-4D2B-89DA-D3D1A63B1B02}.jpg</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>36.21555630555556</v>
+        <v>36.19835088888888</v>
       </c>
       <c r="C40" t="n">
-        <v>36.1609224</v>
+        <v>36.15251038888889</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>{EE051ED5-8815-4C5A-9044-1C37D8094737}.jpg</t>
+          <t>{BD037D65-F49F-4928-9886-8C903F336B99}.jpg</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>36.19660688888889</v>
+        <v>36.21493561111112</v>
       </c>
       <c r="C41" t="n">
-        <v>36.14767</v>
+        <v>36.15828919444444</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>{413B2715-7F2A-4709-8956-064FEA2D5AF0}.jpg</t>
+          <t>{83A27DD6-A1E4-4A52-B89B-33EA3E12EAE2}.jpg</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>37.76664772222222</v>
+        <v>36.21117308333334</v>
       </c>
       <c r="C42" t="n">
-        <v>38.27008745</v>
+        <v>36.14328265555555</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>{E6FCFF1F-B62C-4345-9A86-900E364AC327}.jpg</t>
+          <t>{4E66CC9B-DCB4-404C-B9E3-23DF6CE285C3}.jpg</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>36.21560061111111</v>
+        <v>37.57212277777778</v>
       </c>
       <c r="C43" t="n">
-        <v>36.1403286</v>
+        <v>36.93805176944444</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>{280CB9DC-46D8-4DDD-9910-A0DBAC6E079A}.jpg</t>
+          <t>{08093F3E-19B2-48AE-9016-EE21BA251891}.jpg</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>37.76924633055555</v>
+        <v>36.21840556666667</v>
       </c>
       <c r="C44" t="n">
-        <v>38.26366952777778</v>
+        <v>36.14167557222222</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>{6C7C5BA8-7A25-4537-85ED-46A171F702C6}.jpg</t>
+          <t>{DE318F6C-D145-4768-8B74-A395A7F008BF}.jpg</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>36.19630394444444</v>
+        <v>37.57521897222222</v>
       </c>
       <c r="C45" t="n">
-        <v>36.15433265</v>
+        <v>36.93391122611111</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>{BE32E2E9-8598-457A-AC40-94DE5C1BFC47}.jpg</t>
+          <t>{26BF184B-1422-4604-AEE8-BD8659DF54AA}.jpg</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>37.76414308333333</v>
+        <v>37.57328791666667</v>
       </c>
       <c r="C46" t="n">
-        <v>38.27738761111111</v>
+        <v>36.919614</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>{40945DE5-094B-41DC-9118-34D0AC687B26}.jpg</t>
+          <t>{A0E9FC65-1668-4425-95A2-92754032167E}.jpg</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>36.20477416111111</v>
+        <v>37.76592977777778</v>
       </c>
       <c r="C47" t="n">
-        <v>36.15951838888888</v>
+        <v>38.26638852777778</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>{6B3B4F05-418D-4318-80A0-67FEEE51669C}.jpg</t>
+          <t>{187D9D93-53CC-4953-B80F-3A5107A7192D}.jpg</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>36.23060205555556</v>
+        <v>36.25969455555555</v>
       </c>
       <c r="C48" t="n">
-        <v>36.19999630555555</v>
+        <v>36.20641123888889</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>{068A4180-C955-40E0-B385-BFC75D3C9354}.jpg</t>
+          <t>{D1AD5CAC-68F7-4447-B32D-4155C22BC087}.jpg</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>36.19594633333333</v>
+        <v>37.75662058333333</v>
       </c>
       <c r="C49" t="n">
-        <v>36.15921941666667</v>
+        <v>38.24547044444444</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>{DE318F6C-D145-4768-8B74-A395A7F008BF}.jpg</t>
+          <t>{52F3CCD8-4205-48B5-BDD3-700E4C072A59}.jpg</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>37.57521897222222</v>
+        <v>37.76945910555555</v>
       </c>
       <c r="C50" t="n">
-        <v>36.93391122611111</v>
+        <v>38.26838568888889</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>{B13E60C2-7DF5-47D0-9057-E7AD84699544}.jpg</t>
+          <t>{F0EF1E9D-1E57-47FC-8439-244452934513}.jpg</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>37.76191227777777</v>
+        <v>36.19645522222222</v>
       </c>
       <c r="C51" t="n">
-        <v>38.29055369444444</v>
+        <v>36.16005752777777</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>{41468389-970A-4898-B53E-D4BF30729BB9}.jpg</t>
+          <t>{EB3FE8BD-3F49-484B-892B-4FA8CEA26DAD}.jpg</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>36.22845608333333</v>
+        <v>36.22749417777778</v>
       </c>
       <c r="C52" t="n">
-        <v>36.19931422222222</v>
+        <v>36.166682601</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>{56505110-B3B3-4565-A085-6AB8FF6D1465}.jpg</t>
+          <t>{6888CD02-BE06-4B52-BC8A-098FF1F58E27}.jpg</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>36.21604819444445</v>
+        <v>37.57722222222223</v>
       </c>
       <c r="C53" t="n">
-        <v>36.15878076666667</v>
+        <v>36.91805555555555</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>{4C7C358A-01A7-434B-BDBC-8F459120ACD5}.jpg</t>
+          <t>{B72E134E-3779-4EB8-9C30-42E284F8E511}.jpg</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>36.25973694444444</v>
+        <v>37.57437756666667</v>
       </c>
       <c r="C54" t="n">
-        <v>36.20640348888889</v>
+        <v>36.93379684527778</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>{A5017821-F45A-4FFF-A6DF-BEC41194A5E8}.jpg</t>
+          <t>{7BC03BE0-EBB4-4F80-850D-B1D3F41C7602}.jpg</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>36.2110281</v>
+        <v>36.22872155555556</v>
       </c>
       <c r="C55" t="n">
-        <v>36.16153019444445</v>
+        <v>36.15095917777778</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>{26BF184B-1422-4604-AEE8-BD8659DF54AA}.jpg</t>
+          <t>{5763B662-63E9-43B5-AF81-2611592CF79E}.jpg</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>37.57328791666667</v>
+        <v>36.21973881388889</v>
       </c>
       <c r="C56" t="n">
-        <v>36.919614</v>
+        <v>36.160826</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>{E1038CCD-0C6D-4E1E-A89F-4AF5F7B06564}.jpg</t>
+          <t>{280CB9DC-46D8-4DDD-9910-A0DBAC6E079A}.jpg</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>37.76154788888889</v>
+        <v>37.76924633055555</v>
       </c>
       <c r="C57" t="n">
-        <v>38.24128419444445</v>
+        <v>38.26366952777778</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>{9E270B5D-22BB-4F5B-A895-962198E7C09A}.jpg</t>
+          <t>{A257A9FE-77C2-45EC-891E-9DC249A30005}.jpg</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>37.76945508333333</v>
+        <v>37.57474166666667</v>
       </c>
       <c r="C58" t="n">
-        <v>38.26309669444444</v>
+        <v>36.93337166666667</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>{5763B662-63E9-43B5-AF81-2611592CF79E}.jpg</t>
+          <t>{B80ACF18-864C-4E62-BB4A-56820D4621C7}.jpg</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>36.21973881388889</v>
+        <v>36.19611305555555</v>
       </c>
       <c r="C59" t="n">
-        <v>36.160826</v>
+        <v>36.15939951666667</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>{E65D3BBF-2079-4F2D-B18E-712F323ECEB5}.jpg</t>
+          <t>{CA3CF42C-1BAC-4300-8942-CF049F944ABD}.jpg</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>37.59701713888889</v>
+        <v>36.21773038888889</v>
       </c>
       <c r="C60" t="n">
-        <v>36.86324386111112</v>
+        <v>36.15750787222222</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>{4811BD15-A31A-4D98-823C-A498A1739210}.jpg</t>
+          <t>{140D61AC-0E19-4134-8EF7-656DB1323C44}.jpg</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>37.58880768055556</v>
+        <v>36.49513530555556</v>
       </c>
       <c r="C61" t="n">
-        <v>36.88633386111111</v>
+        <v>36.36784786944445</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>{84DD3BE8-91B0-46CF-BEFF-3F6800C0E00A}.jpg</t>
+          <t>{9CB58159-DB90-4641-BAAE-DA7D123CF1CA}.jpg</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>36.20644661111111</v>
+        <v>36.21722031305556</v>
       </c>
       <c r="C62" t="n">
-        <v>36.15896394444444</v>
+        <v>36.15681531666667</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>{E316E926-E8EE-4EA4-B951-0736886C9B20}.jpg</t>
+          <t>{8ABA5D32-68F5-4B8C-8E2B-33335818C3A6}.jpg</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>37.55946666666667</v>
+        <v>36.2157633888889</v>
       </c>
       <c r="C63" t="n">
-        <v>36.9209</v>
+        <v>36.1574949</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>{5E6BD6EA-F129-410F-9C93-13D4DE27771C}.jpg</t>
+          <t>{9AEB2EA6-67A4-402D-86DF-66F3AD34A946}.jpg</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>37.57328694444445</v>
+        <v>37.76503930555555</v>
       </c>
       <c r="C64" t="n">
-        <v>36.91925611944444</v>
+        <v>38.2371118</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>{BE11E2F6-7A43-4B94-B9E4-76959ABEB005}.jpg</t>
+          <t>{80EAEDD9-1807-45E1-88AD-55006C712D03}.jpg</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>37.57227643055556</v>
+        <v>37.76325691666667</v>
       </c>
       <c r="C65" t="n">
-        <v>36.93743236111111</v>
+        <v>38.28148530555556</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>{2E8A4D8B-4402-411B-BC72-055629FBD782}.jpg</t>
+          <t>{78FAE855-EC87-49CD-BEDC-A7B036B51976}.jpg</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>36.20669783333334</v>
+        <v>36.23594945</v>
       </c>
       <c r="C66" t="n">
-        <v>36.15879837777778</v>
+        <v>36.16806895833333</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>{6C828523-2706-438A-8990-46EEBAE0D62D}.jpg</t>
+          <t>{246A5A81-F042-4258-A6C2-A4F061E2D0BB}.jpg</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>36.22010585555556</v>
+        <v>36.22787969444445</v>
       </c>
       <c r="C67" t="n">
-        <v>36.15710308333333</v>
+        <v>36.14938769444444</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>{975C5CBA-9329-4F97-88D8-4B156D764FF6}.jpg</t>
+          <t>{32E8B3F6-1A3C-40F6-AFB2-2B0C2C0428B4}.jpg</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>36.2188823</v>
+        <v>36.19795125</v>
       </c>
       <c r="C68" t="n">
-        <v>36.1620305</v>
+        <v>36.16537925</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>{787702D3-C98A-4B4F-809D-23B8358B4666}.jpg</t>
+          <t>{1A1C3737-55C9-4D47-80D8-71E9A3C90F97}.jpg</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>37.76055713888889</v>
+        <v>36.49511380555555</v>
       </c>
       <c r="C69" t="n">
-        <v>38.24986230555556</v>
+        <v>36.36793245</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>{BE7EAED6-A6CD-41E4-B5FD-B5AD329A4363}.jpg</t>
+          <t>{A270F1A2-971F-4949-9F24-96DB5E508FF0}.jpg</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>37.68665833333333</v>
+        <v>37.76482141666666</v>
       </c>
       <c r="C70" t="n">
-        <v>37.86949350833333</v>
+        <v>38.27756212222222</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>{C2EEF875-FCC6-4CF2-A186-334FFC456E56}.jpg</t>
+          <t>{967714B1-CD17-4C6D-B5C4-D669E2664BD2}.jpg</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>36.25975455555555</v>
+        <v>36.22918972222222</v>
       </c>
       <c r="C71" t="n">
-        <v>36.20638661944444</v>
+        <v>36.16778296388889</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>{6888CD02-BE06-4B52-BC8A-098FF1F58E27}.jpg</t>
+          <t>{64168C52-3BE4-43EA-8E3B-0999F05147AC}.jpg</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>37.57722222222223</v>
+        <v>36.20614769444445</v>
       </c>
       <c r="C72" t="n">
-        <v>36.91805555555555</v>
+        <v>36.15642387777778</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>{967714B1-CD17-4C6D-B5C4-D669E2664BD2}.jpg</t>
+          <t>{29D9B737-344B-40CC-B959-D2305A84A668}.jpg</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>36.22918972222222</v>
+        <v>36.19824191666666</v>
       </c>
       <c r="C73" t="n">
-        <v>36.16778296388889</v>
+        <v>36.16050406944444</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>{93CA0A7E-EF3F-43AC-BE9B-5C7EE7DBC5E7}.jpg</t>
+          <t>{A9078FAA-C0C7-4EB0-87EB-2D936A70B2CA}.jpg</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>36.49920605555555</v>
+        <v>37.68828020555555</v>
       </c>
       <c r="C74" t="n">
-        <v>36.34610094444444</v>
+        <v>37.85578821388889</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>{E52E9E22-3D04-47B6-A1C7-62C91B1A2F2D}.jpg</t>
+          <t>{EC63F45D-EE35-4AB7-8652-339A19EC0235}.jpg</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>36.56528158333333</v>
+        <v>37.752323</v>
       </c>
       <c r="C75" t="n">
-        <v>36.15630683888889</v>
+        <v>38.24599119444444</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>{54C29DE1-D371-4A72-801B-97570E29D5BC}.jpg</t>
+          <t>{DB865BB7-D755-4775-BCBE-013D69FF57EB}.jpg</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>37.76448388888889</v>
+        <v>37.57518</v>
       </c>
       <c r="C76" t="n">
-        <v>38.2355288</v>
+        <v>36.933075</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>{C3283350-EC30-4BE6-B17C-BAC34AAE6747}.jpg</t>
+          <t>{82C32338-B145-4825-8515-E49CDDE68032}.jpg</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>37.57517511111111</v>
+        <v>36.23181541666667</v>
       </c>
       <c r="C77" t="n">
-        <v>36.93200433333333</v>
+        <v>36.16548463888888</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>{56399E0B-86C8-4C7E-8446-A9B9CDF05158}.jpg</t>
+          <t>{6A6ED554-4709-4BDA-9709-BECEB8F41628}.jpg</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>37.76356580555556</v>
+        <v>37.57207012777778</v>
       </c>
       <c r="C78" t="n">
-        <v>38.24116580555555</v>
+        <v>36.92389843055555</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>{F4FC4A8F-455C-4FE4-8EC1-5A90CDA778F0}.jpg</t>
+          <t>{E31AE50A-1982-4A70-B59B-424B598D1A40}.jpg</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>36.20707975000001</v>
+        <v>36.2173728</v>
       </c>
       <c r="C79" t="n">
-        <v>36.15848142777778</v>
+        <v>36.17171579999999</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>{F9E69747-3A8E-4D2B-89DA-D3D1A63B1B02}.jpg</t>
+          <t>{FF3046E1-7C71-44D6-BDBF-21E92799D7E1}.jpg</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>36.19835088888888</v>
+        <v>36.22242430555556</v>
       </c>
       <c r="C80" t="n">
-        <v>36.15251038888889</v>
+        <v>36.1543973</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>{D593BFFF-7803-49A3-9973-883F1A3DD122}.jpg</t>
+          <t>{4C7C358A-01A7-434B-BDBC-8F459120ACD5}.jpg</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>37.7638975</v>
+        <v>36.25973694444444</v>
       </c>
       <c r="C81" t="n">
-        <v>38.27213311111111</v>
+        <v>36.20640348888889</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>{CD574077-0E65-4263-8E08-DF099D9B31B4}.jpg</t>
+          <t>{068A4180-C955-40E0-B385-BFC75D3C9354}.jpg</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>36.20633603611111</v>
+        <v>36.19594633333333</v>
       </c>
       <c r="C82" t="n">
-        <v>36.15694974166666</v>
+        <v>36.15921941666667</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>{FAEB5345-2C23-4AF0-8A3F-3B5D19D14C64}.jpg</t>
+          <t>{6806A4A9-CD94-4360-B74D-83BF39DAF537}.jpg</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>37.55962666666667</v>
+        <v>36.21795554444444</v>
       </c>
       <c r="C83" t="n">
-        <v>36.92028999999999</v>
+        <v>36.15632415555555</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>{29D9B737-344B-40CC-B959-D2305A84A668}.jpg</t>
+          <t>{1D8F887A-9D75-448A-87A8-33AEBC6ABFB4}.jpg</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>36.19824191666666</v>
+        <v>37.5718793888889</v>
       </c>
       <c r="C84" t="n">
-        <v>36.16050406944444</v>
+        <v>36.92210701944444</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>{992B9E79-CF5B-44F7-B2C3-9F0D28A1A12E}.jpg</t>
+          <t>{6C828523-2706-438A-8990-46EEBAE0D62D}.jpg</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>36.25974716666666</v>
+        <v>36.22010585555556</v>
       </c>
       <c r="C85" t="n">
-        <v>36.20638947222223</v>
+        <v>36.15710308333333</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>{D68EFBBB-8DFB-4F02-930D-AE9DDBDE858F}.jpg</t>
+          <t>{2E8A4D8B-4402-411B-BC72-055629FBD782}.jpg</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>36.20416505555556</v>
+        <v>36.20669783333334</v>
       </c>
       <c r="C86" t="n">
-        <v>36.14976594444445</v>
+        <v>36.15879837777778</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>{CCE1D552-EEA7-4EB0-B337-B91E6357B702}.jpg</t>
+          <t>{7A50EFD3-041C-4575-B53F-294A71AF3D6D}.jpg</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>36.25973426111111</v>
+        <v>37.76694979527777</v>
       </c>
       <c r="C87" t="n">
-        <v>36.20640416111112</v>
+        <v>38.26132027777778</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>{FE9A1FE9-65C1-4CF4-A574-5F893E070206}.jpg</t>
+          <t>{5BA2AAD0-5AE3-4261-9233-4E241D59B065}.jpg</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>36.19766158333333</v>
+        <v>36.22861575</v>
       </c>
       <c r="C88" t="n">
-        <v>36.15319432777778</v>
+        <v>36.19683311111111</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>{780461B9-3366-430D-BF71-0340723D371F}.jpg</t>
+          <t>{13B0F93E-52A9-4884-AFC5-661AC641A905}.jpg</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>36.21637075</v>
+        <v>37.75872943055555</v>
       </c>
       <c r="C89" t="n">
-        <v>36.15504469444444</v>
+        <v>38.26542552777778</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>{722D2712-501F-4188-9BD8-636D6F3B30CA}.jpg</t>
+          <t>{7E845995-5476-43EA-A08F-0AEB26D8E996}.jpg</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>37.57521922222222</v>
+        <v>36.20154177222223</v>
       </c>
       <c r="C90" t="n">
-        <v>36.93391326944444</v>
+        <v>36.16488152777777</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>{1F4AE99E-2294-417D-819B-FE3902ECF50E}.jpg</t>
+          <t>{F180F6DF-60C9-483C-A4E8-679B207DB9A7}.jpg</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>36.2597146</v>
+        <v>36.19751488888888</v>
       </c>
       <c r="C91" t="n">
-        <v>36.20639751944444</v>
+        <v>36.16060378888888</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>{30682C10-CC92-48E0-9BD0-5D85C1648D89}.jpg</t>
+          <t>{08CD4653-870D-4E6A-8D26-CD71C982C3D1}.jpg</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>36.19593288888888</v>
+        <v>36.23115022222223</v>
       </c>
       <c r="C92" t="n">
-        <v>36.16002119444444</v>
+        <v>36.19971825</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>{340592C4-441E-4BB9-AFA9-796650C22585}.jpg</t>
+          <t>{C3F83540-E59B-422E-A604-15DE93CE76DD}.jpg</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>36.20312220277778</v>
+        <v>37.06308333333333</v>
       </c>
       <c r="C93" t="n">
-        <v>36.15145024444444</v>
+        <v>36.23664444444444</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>{765D8073-D876-436E-9F71-865579FC3ABF}.jpg</t>
+          <t>{E6F5A316-85F0-4566-978A-18CCD49F1DC3}.jpg</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>37.76478130555556</v>
+        <v>37.76822578055555</v>
       </c>
       <c r="C94" t="n">
-        <v>38.27818677777778</v>
+        <v>38.26071347222222</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>{4AD3B275-A164-4918-9993-06F17A29CB18}.jpg</t>
+          <t>{1FD1218E-ACF9-40D0-B4B4-106C37BD8878}.jpg</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>37.76141666666667</v>
+        <v>37.57193877777778</v>
       </c>
       <c r="C95" t="n">
-        <v>38.26574166666666</v>
+        <v>36.91998378888889</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>{55E6D05F-34D4-4933-8676-3C22C672929E}.jpg</t>
+          <t>{F6CA6BB0-293B-43A4-9C62-53F015D6A646}.jpg</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>37.76337769444444</v>
+        <v>37.58136727777778</v>
       </c>
       <c r="C96" t="n">
-        <v>38.24220380555555</v>
+        <v>36.96623416666667</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>{0F98F3F0-1AE5-4434-AD6A-A2613F4F2664}.jpg</t>
+          <t>{E65D3BBF-2079-4F2D-B18E-712F323ECEB5}.jpg</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>37.74781297222222</v>
+        <v>37.59701713888889</v>
       </c>
       <c r="C97" t="n">
-        <v>38.24954358333333</v>
+        <v>36.86324386111112</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>{0B7CEF9B-C3E6-43C1-BF94-FB1C04A984E6}.jpg</t>
+          <t>{907FEA05-9978-418E-923A-006E5907B677}.jpg</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>37.77358399166667</v>
+        <v>37.57328095277778</v>
       </c>
       <c r="C98" t="n">
-        <v>38.26891006388889</v>
+        <v>36.91966454444444</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>{DD895B74-E3FC-470D-8937-50E3DEF4AC9A}.jpg</t>
+          <t>{0F98F3F0-1AE5-4434-AD6A-A2613F4F2664}.jpg</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>37.57142725000001</v>
+        <v>37.74781297222222</v>
       </c>
       <c r="C99" t="n">
-        <v>36.936136875</v>
+        <v>38.24954358333333</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>{1A8FF8A6-63FE-4F2F-99FF-CD4B1E3DD047}.jpg</t>
+          <t>{C79931AC-1A1F-4906-8761-5E276EC978EF}.jpg</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>36.23682021111111</v>
+        <v>36.23457488055556</v>
       </c>
       <c r="C100" t="n">
-        <v>36.165431</v>
+        <v>36.16567141666666</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>{89A572CB-D830-4737-BB40-A0597F77CB72}.jpg</t>
+          <t>{0F20EE24-A6F5-434A-A8BC-A69A2233D152}.jpg</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>37.58176808333334</v>
+        <v>36.20747659166667</v>
       </c>
       <c r="C101" t="n">
-        <v>36.96571811111112</v>
+        <v>36.15842320555556</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>{5F0DDCA3-02B8-4FED-A838-88FCF36D1F74}.jpg</t>
+          <t>{09B0A8BE-FC31-4BCD-9286-E6C3D6D4E400}.jpg</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>37.7663325</v>
+        <v>36.23008572222222</v>
       </c>
       <c r="C102" t="n">
-        <v>38.26236283333333</v>
+        <v>36.14873766666667</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>{93C31A94-5FB3-4199-9685-EECC1833BC93}.jpg</t>
+          <t>{BC1D7E63-7E14-49A5-BDE9-A4FF91774D7D}.jpg</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>37.76993075277777</v>
+        <v>36.21394394444444</v>
       </c>
       <c r="C103" t="n">
-        <v>38.26451266666667</v>
+        <v>36.16930606111111</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>{E851A14E-6C4F-4FA0-95FF-18957BE4EFE1}.jpg</t>
+          <t>{722D2712-501F-4188-9BD8-636D6F3B30CA}.jpg</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>37.76634361111111</v>
+        <v>37.57521922222222</v>
       </c>
       <c r="C104" t="n">
-        <v>38.27160925</v>
+        <v>36.93391326944444</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>{A7FA99B1-A07B-42D6-AD97-53EBB6227CBD}.jpg</t>
+          <t>{F344DA1B-45CB-4B77-B323-ADF7FF9A0C58}.jpg</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>37.68800143888888</v>
+        <v>37.58327927777778</v>
       </c>
       <c r="C105" t="n">
-        <v>37.85607461944445</v>
+        <v>36.96482725000001</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>{533D50D1-37C8-4C1D-8FBE-6BA7CCA620AF}.jpg</t>
+          <t>{CBA5B01F-FA8C-4FD0-AC71-94406D789E9B}.jpg</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>37.57157127222222</v>
+        <v>37.57385127777778</v>
       </c>
       <c r="C106" t="n">
-        <v>36.93660743888888</v>
+        <v>36.93466128888888</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>{5A3A809A-E6C7-4A7B-97D2-C071B20C1416}.jpg</t>
+          <t>{E6FCFF1F-B62C-4345-9A86-900E364AC327}.jpg</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>37.771418625</v>
+        <v>36.21560061111111</v>
       </c>
       <c r="C107" t="n">
-        <v>38.26922974444444</v>
+        <v>36.1403286</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>{E536BE4A-A604-4313-BC64-2876374E677F}.jpg</t>
+          <t>{1F4AE99E-2294-417D-819B-FE3902ECF50E}.jpg</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>37.76464019444445</v>
+        <v>36.2597146</v>
       </c>
       <c r="C108" t="n">
-        <v>38.27032038055555</v>
+        <v>36.20639751944444</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>{18E93204-2591-4C7D-BBBC-BB39F5E7BE50}.jpg</t>
+          <t>{70CDA7EC-DA54-4EC9-9ABA-A35F84F6B4F3}.jpg</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>36.19602124999999</v>
+        <v>36.2058461</v>
       </c>
       <c r="C109" t="n">
-        <v>36.15823852777778</v>
+        <v>36.159881</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>{26BCBA63-E13F-4E7B-A019-BE7A4C63A053}.jpg</t>
+          <t>{FE9A1FE9-65C1-4CF4-A574-5F893E070206}.jpg</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>37.570865</v>
+        <v>36.19766158333333</v>
       </c>
       <c r="C110" t="n">
-        <v>36.91841333333333</v>
+        <v>36.15319432777778</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>{76385D9D-0839-4B82-ADF6-F3318D1EF23F}.jpg</t>
+          <t>{9FED06B1-A2CE-4106-87D7-6B4CB6D55CCA}.jpg</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>37.57472775</v>
+        <v>36.20873725000001</v>
       </c>
       <c r="C111" t="n">
-        <v>36.94820544444444</v>
+        <v>36.15536491666666</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>{3D4584B3-BE53-46C0-BB59-D8A9D355B08A}.jpg</t>
+          <t>{684586A6-5FE3-4604-9A55-31F094D3541B}.jpg</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>36.23589883333334</v>
+        <v>36.19468390277778</v>
       </c>
       <c r="C112" t="n">
-        <v>36.16497836111111</v>
+        <v>36.14500444444445</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>{8CBE25CB-016C-4B12-AFA7-AAEFCAE027E6}.jpg</t>
+          <t>{765D8073-D876-436E-9F71-865579FC3ABF}.jpg</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>36.21739308166667</v>
+        <v>37.76478130555556</v>
       </c>
       <c r="C113" t="n">
-        <v>36.15651826388888</v>
+        <v>38.27818677777778</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>{2A00B94E-8B01-4342-8E9E-6E3DEFAD2B09}.jpg</t>
+          <t>{220782BB-3CED-4B7C-B1F9-5C55C0545FD2}.jpg</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>37.75638319444445</v>
+        <v>37.76109163888889</v>
       </c>
       <c r="C114" t="n">
-        <v>38.2355974</v>
+        <v>38.25722463888889</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>{684586A6-5FE3-4604-9A55-31F094D3541B}.jpg</t>
+          <t>{8C45868F-979A-432F-8C42-4B0DEFA80225}.jpg</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>36.19468390277778</v>
+        <v>36.20622158333334</v>
       </c>
       <c r="C115" t="n">
-        <v>36.14500444444445</v>
+        <v>36.17344077777778</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>{EECF3874-303B-44C7-A044-8C7A2308204B}.jpg</t>
+          <t>{84DD3BE8-91B0-46CF-BEFF-3F6800C0E00A}.jpg</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>36.19847755555555</v>
+        <v>36.20644661111111</v>
       </c>
       <c r="C116" t="n">
-        <v>36.15426723055555</v>
+        <v>36.15896394444444</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>{B8C22D59-9E12-478E-A174-EF310DCDA7C1}.jpg</t>
+          <t>{4C0E89B0-626A-42D6-BB95-03ABF20E6B8D}.jpg</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>36.19422536111111</v>
+        <v>36.21713776305555</v>
       </c>
       <c r="C117" t="n">
-        <v>36.15166751111111</v>
+        <v>36.15580826944444</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>{81941BBB-5130-47D0-8A5E-F39E9BC214A8}.jpg</t>
+          <t>{50ABCC39-1DB7-4A13-944E-53EAB603ED2E}.jpg</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>36.21663263888889</v>
+        <v>36.21288877777778</v>
       </c>
       <c r="C118" t="n">
-        <v>36.16098418333333</v>
+        <v>36.14085708333333</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>{902AF0E6-0DC8-4F1C-BAD3-A44A382DB66F}.jpg</t>
+          <t>{B8C22D59-9E12-478E-A174-EF310DCDA7C1}.jpg</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>37.76309269444445</v>
+        <v>36.19422536111111</v>
       </c>
       <c r="C119" t="n">
-        <v>38.2394074</v>
+        <v>36.15166751111111</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>{4EB7C352-B021-4451-B8F3-074B91C51ADD}.jpg</t>
+          <t>{454A120C-20F7-499F-9CA3-70C771A7FD3A}.jpg</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>37.68755141666666</v>
+        <v>36.20568175</v>
       </c>
       <c r="C120" t="n">
-        <v>37.82890505555556</v>
+        <v>36.15529327777778</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>{B2B3C2E9-5A4C-4889-BCC2-38A29B3300C8}.jpg</t>
+          <t>{451DBC30-C4F6-4961-8B2D-D223D5B3D20C}.jpg</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>36.19560213888889</v>
+        <v>36.19433488888888</v>
       </c>
       <c r="C121" t="n">
-        <v>36.15956888888888</v>
+        <v>36.15159435</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>{6FFEFA7D-F17D-4627-B55D-3CD949C486D3}.jpg</t>
+          <t>{1E214BAA-AEE7-41AE-90B3-8E1C6D0FBB29}.jpg</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>36.20325993055556</v>
+        <v>36.25973786111111</v>
       </c>
       <c r="C122" t="n">
-        <v>36.14778175</v>
+        <v>36.20640465</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>{16C2E690-76CF-4A5E-B8A6-6E1AEAB58D1C}.jpg</t>
+          <t>{4EB7C352-B021-4451-B8F3-074B91C51ADD}.jpg</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>37.77255085277778</v>
+        <v>37.68755141666666</v>
       </c>
       <c r="C123" t="n">
-        <v>38.26293702777778</v>
+        <v>37.82890505555556</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>{5F85BE1A-EE78-4FD7-8F28-C95BAD00EFB1}.jpg</t>
+          <t>{7131FB9E-B9E7-4612-8926-04EFF43110E2}.jpg</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>37.57198225</v>
+        <v>37.76333980555555</v>
       </c>
       <c r="C124" t="n">
-        <v>36.93414867583333</v>
+        <v>38.2421846</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>{82E413CE-B196-4D2B-9CA7-60ACA26BA5E6}.jpg</t>
+          <t>{BE11E2F6-7A43-4B94-B9E4-76959ABEB005}.jpg</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>37.75567783888889</v>
+        <v>37.57227643055556</v>
       </c>
       <c r="C125" t="n">
-        <v>38.26574125</v>
+        <v>36.93743236111111</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>{96ECEBEC-678F-4D8B-A811-CBD3D830280C}.jpg</t>
+          <t>{136B3821-143F-4048-BF13-D14D0CA38227}.jpg</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>36.23134569444445</v>
+        <v>36.21555630555556</v>
       </c>
       <c r="C126" t="n">
-        <v>36.16525444444444</v>
+        <v>36.1609224</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>{EB3FE8BD-3F49-484B-892B-4FA8CEA26DAD}.jpg</t>
+          <t>{0B7CEF9B-C3E6-43C1-BF94-FB1C04A984E6}.jpg</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>36.22749417777778</v>
+        <v>37.77358399166667</v>
       </c>
       <c r="C127" t="n">
-        <v>36.166682601</v>
+        <v>38.26891006388889</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>{8323814C-3708-4EAB-B5B7-B6B0B2B9CB96}.jpg</t>
+          <t>{2A8304E5-B65C-4A49-A745-FD29854CEC7A}.jpg</t>
         </is>
       </c>
       <c r="B128" t="n">
-        <v>37.73547438333333</v>
+        <v>37.7519047</v>
       </c>
       <c r="C128" t="n">
-        <v>38.223239</v>
+        <v>38.24508180555556</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>{B91E6057-C51E-4712-AE63-EA2D8CC1E02B}.jpg</t>
+          <t>{4B067E7F-6299-4C82-A2A3-F9903425355B}.jpg</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>36.23151038888889</v>
+        <v>36.20492681111111</v>
       </c>
       <c r="C129" t="n">
-        <v>36.16660011111111</v>
+        <v>36.15883581666667</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>{1243072D-C509-4AD1-BE81-83F18A77CB71}.jpg</t>
+          <t>{C3A58B21-AD3A-4596-82EF-1D27DEA064C1}.jpg</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>36.19771411111111</v>
+        <v>36.25972444444444</v>
       </c>
       <c r="C130" t="n">
-        <v>36.1636545</v>
+        <v>36.20637865</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>{CBA5B01F-FA8C-4FD0-AC71-94406D789E9B}.jpg</t>
+          <t>{2E93A44B-A3F3-44D8-BC4B-6B0D877F2729}.jpg</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>37.57385127777778</v>
+        <v>36.2313595</v>
       </c>
       <c r="C131" t="n">
-        <v>36.93466128888888</v>
+        <v>36.16506752777778</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>{0F2ADD6B-076F-4A45-B91D-7C63B32CB26F}.jpg</t>
+          <t>{A5017821-F45A-4FFF-A6DF-BEC41194A5E8}.jpg</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>36.20645642777778</v>
+        <v>36.2110281</v>
       </c>
       <c r="C132" t="n">
-        <v>36.15686209722222</v>
+        <v>36.16153019444445</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>{396528FE-159B-4406-AF75-9EE1279E7ED9}.jpg</t>
+          <t>{CBC9BA7D-56F2-4628-ADF1-235F4D89B84C}.jpg</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>37.76869134444444</v>
+        <v>36.19663611111111</v>
       </c>
       <c r="C133" t="n">
-        <v>38.26108356944444</v>
+        <v>36.14903888888889</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>{A289263E-4C12-4525-ADAB-E912A19D1D58}.jpg</t>
+          <t>{64F928F8-E576-42EC-B868-2AC2609D1CB5}.jpg</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>37.56425166666666</v>
+        <v>37.57297852777778</v>
       </c>
       <c r="C134" t="n">
-        <v>36.921615</v>
+        <v>36.93573819166667</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>{1A1C3737-55C9-4D47-80D8-71E9A3C90F97}.jpg</t>
+          <t>{18E93204-2591-4C7D-BBBC-BB39F5E7BE50}.jpg</t>
         </is>
       </c>
       <c r="B135" t="n">
-        <v>36.49511380555555</v>
+        <v>36.19602124999999</v>
       </c>
       <c r="C135" t="n">
-        <v>36.36793245</v>
+        <v>36.15823852777778</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>{7A50EFD3-041C-4575-B53F-294A71AF3D6D}.jpg</t>
+          <t>{3CEF804A-20EB-4D03-9DFB-B5D29F4A7542}.jpg</t>
         </is>
       </c>
       <c r="B136" t="n">
-        <v>37.76694979527777</v>
+        <v>36.2111895</v>
       </c>
       <c r="C136" t="n">
-        <v>38.26132027777778</v>
+        <v>36.16153138888889</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>{70CDA7EC-DA54-4EC9-9ABA-A35F84F6B4F3}.jpg</t>
+          <t>{FE961C6B-6B7A-4D76-9A8F-AE33749201C2}.jpg</t>
         </is>
       </c>
       <c r="B137" t="n">
-        <v>36.2058461</v>
+        <v>36.22756836111111</v>
       </c>
       <c r="C137" t="n">
-        <v>36.159881</v>
+        <v>36.15120042777777</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>{DB865BB7-D755-4775-BCBE-013D69FF57EB}.jpg</t>
+          <t>{6AF44EB2-4F33-44F6-82BD-E746DE95516C}.jpg</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>37.57518</v>
+        <v>36.206336575</v>
       </c>
       <c r="C138" t="n">
-        <v>36.933075</v>
+        <v>36.15693163888889</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>{CA244B31-8A24-423D-82B4-91FA2E8A0D84}.jpg</t>
+          <t>{292912A9-674E-4A41-89DD-7F0E0E550A84}.jpg</t>
         </is>
       </c>
       <c r="B139" t="n">
-        <v>37.59167218055556</v>
+        <v>37.78029586111111</v>
       </c>
       <c r="C139" t="n">
-        <v>36.86593441666667</v>
+        <v>38.25637026944445</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>{2E93A44B-A3F3-44D8-BC4B-6B0D877F2729}.jpg</t>
+          <t>{CA244B31-8A24-423D-82B4-91FA2E8A0D84}.jpg</t>
         </is>
       </c>
       <c r="B140" t="n">
-        <v>36.2313595</v>
+        <v>37.59167218055556</v>
       </c>
       <c r="C140" t="n">
-        <v>36.16506752777778</v>
+        <v>36.86593441666667</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>{ECF3A29B-3481-4627-89C9-1595B4880DD2}.jpg</t>
+          <t>{BE7EAED6-A6CD-41E4-B5FD-B5AD329A4363}.jpg</t>
         </is>
       </c>
       <c r="B141" t="n">
-        <v>37.7531797</v>
+        <v>37.68665833333333</v>
       </c>
       <c r="C141" t="n">
-        <v>38.24628711111112</v>
+        <v>37.86949350833333</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>{F344DA1B-45CB-4B77-B323-ADF7FF9A0C58}.jpg</t>
+          <t>{4811BD15-A31A-4D98-823C-A498A1739210}.jpg</t>
         </is>
       </c>
       <c r="B142" t="n">
-        <v>37.58327927777778</v>
+        <v>37.58880768055556</v>
       </c>
       <c r="C142" t="n">
-        <v>36.96482725000001</v>
+        <v>36.88633386111111</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>{D9FC1386-FE62-42FD-A745-F5537968F51B}.jpg</t>
+          <t>{07AD392A-3C05-451D-836E-FED8051022F9}.jpg</t>
         </is>
       </c>
       <c r="B143" t="n">
-        <v>37.76303597222222</v>
+        <v>36.20226519166667</v>
       </c>
       <c r="C143" t="n">
-        <v>38.29036194444444</v>
+        <v>36.1641085</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>{82117B6A-CB2C-456F-9DAA-DBDA8C206503}.jpg</t>
+          <t>{82E413CE-B196-4D2B-9CA7-60ACA26BA5E6}.jpg</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>36.19532788888888</v>
+        <v>37.75567783888889</v>
       </c>
       <c r="C144" t="n">
-        <v>36.15280598888889</v>
+        <v>38.26574125</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>{78FAE855-EC87-49CD-BEDC-A7B036B51976}.jpg</t>
+          <t>{561F2B1A-FA0F-4657-B868-1510ADC53059}.jpg</t>
         </is>
       </c>
       <c r="B145" t="n">
-        <v>36.23594945</v>
+        <v>36.21383997222222</v>
       </c>
       <c r="C145" t="n">
-        <v>36.16806895833333</v>
+        <v>36.15835197222222</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>{60692F62-3CBD-4B7A-B30B-66C3CA72BD9F}.jpg</t>
+          <t>{5F0DDCA3-02B8-4FED-A838-88FCF36D1F74}.jpg</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>36.218100825</v>
+        <v>37.7663325</v>
       </c>
       <c r="C146" t="n">
-        <v>36.15625135555555</v>
+        <v>38.26236283333333</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>{DA075791-5464-410E-AA19-726B5B154045}.jpg</t>
+          <t>{56399E0B-86C8-4C7E-8446-A9B9CDF05158}.jpg</t>
         </is>
       </c>
       <c r="B147" t="n">
-        <v>36.20225089722223</v>
+        <v>37.76356580555556</v>
       </c>
       <c r="C147" t="n">
-        <v>36.14826561111111</v>
+        <v>38.24116580555555</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>{C5F45ECB-2CC0-4F16-91D1-D04B7F0EC49D}.jpg</t>
+          <t>{15FBDDE2-574A-4703-BC41-B676FE4C1B36}.jpg</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>36.22708157222223</v>
+        <v>37.5872535</v>
       </c>
       <c r="C148" t="n">
-        <v>36.16443405555555</v>
+        <v>36.94399566666667</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>{440E99B0-8701-492A-BBC4-5DB76137C7CA}.jpg</t>
+          <t>{DD895B74-E3FC-470D-8937-50E3DEF4AC9A}.jpg</t>
         </is>
       </c>
       <c r="B149" t="n">
-        <v>36.56693796694445</v>
+        <v>37.57142725000001</v>
       </c>
       <c r="C149" t="n">
-        <v>36.15080136305556</v>
+        <v>36.936136875</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>{09BA246A-63EB-4C38-9ED9-CB5A905081B8}.jpg</t>
+          <t>{30682C10-CC92-48E0-9BD0-5D85C1648D89}.jpg</t>
         </is>
       </c>
       <c r="B150" t="n">
-        <v>37.78045788888889</v>
+        <v>36.19593288888888</v>
       </c>
       <c r="C150" t="n">
-        <v>38.25664012777778</v>
+        <v>36.16002119444444</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>{C3F83540-E59B-422E-A604-15DE93CE76DD}.jpg</t>
+          <t>{B1D62FB5-6F0F-408A-BBF3-BF2F64BA5012}.jpg</t>
         </is>
       </c>
       <c r="B151" t="n">
-        <v>37.06308333333333</v>
+        <v>37.76829</v>
       </c>
       <c r="C151" t="n">
-        <v>36.23664444444444</v>
+        <v>38.26105833333333</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>{32E8B3F6-1A3C-40F6-AFB2-2B0C2C0428B4}.jpg</t>
+          <t>{5E830776-FCE1-480F-9B52-9B76D84C0BCD}.jpg</t>
         </is>
       </c>
       <c r="B152" t="n">
-        <v>36.19795125</v>
+        <v>36.2597279</v>
       </c>
       <c r="C152" t="n">
-        <v>36.16537925</v>
+        <v>36.20637535</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>{C3A58B21-AD3A-4596-82EF-1D27DEA064C1}.jpg</t>
+          <t>{ACED80DF-AC07-4AC7-A414-60E43822762C}.jpg</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>36.25972444444444</v>
+        <v>37.77459511111111</v>
       </c>
       <c r="C153" t="n">
-        <v>36.20637865</v>
+        <v>38.26554547222222</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>{A270F1A2-971F-4949-9F24-96DB5E508FF0}.jpg</t>
+          <t>{40945DE5-094B-41DC-9118-34D0AC687B26}.jpg</t>
         </is>
       </c>
       <c r="B154" t="n">
-        <v>37.76482141666666</v>
+        <v>36.20477416111111</v>
       </c>
       <c r="C154" t="n">
-        <v>38.27756212222222</v>
+        <v>36.15951838888888</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>{45A41380-3CD2-45F5-8ADF-F6AC5FA95246}.jpg</t>
+          <t>{C5F45ECB-2CC0-4F16-91D1-D04B7F0EC49D}.jpg</t>
         </is>
       </c>
       <c r="B155" t="n">
-        <v>36.20962196111111</v>
+        <v>36.22708157222223</v>
       </c>
       <c r="C155" t="n">
-        <v>36.16005752777777</v>
+        <v>36.16443405555555</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>{6D52D63A-D29B-415F-B136-FCFDF6BCFFFF}.jpg</t>
+          <t>{D9FC1386-FE62-42FD-A745-F5537968F51B}.jpg</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>36.21747463722222</v>
+        <v>37.76303597222222</v>
       </c>
       <c r="C156" t="n">
-        <v>36.16127780555556</v>
+        <v>38.29036194444444</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>{BBD96776-C4A8-40A8-AEE2-95C783C30AD6}.jpg</t>
+          <t>{96ECEBEC-678F-4D8B-A811-CBD3D830280C}.jpg</t>
         </is>
       </c>
       <c r="B157" t="n">
-        <v>36.21687546861111</v>
+        <v>36.23134569444445</v>
       </c>
       <c r="C157" t="n">
-        <v>36.16106102777778</v>
+        <v>36.16525444444444</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>{C0321E11-988C-4759-BD4F-48BE594C83C0}.jpg</t>
+          <t>{0F27053B-62EE-42CE-AABD-98680EF9C411}.jpg</t>
         </is>
       </c>
       <c r="B158" t="n">
-        <v>37.75964598888889</v>
+        <v>36.22748977777778</v>
       </c>
       <c r="C158" t="n">
-        <v>38.25997297222222</v>
+        <v>36.15124046944445</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>{C17DE65C-762E-41D9-A6FA-CCD9B77F5D62}.jpg</t>
+          <t>{12D329B8-7451-468E-B226-530A2D215515}.jpg</t>
         </is>
       </c>
       <c r="B159" t="n">
-        <v>37.76400797222222</v>
+        <v>36.25971043055556</v>
       </c>
       <c r="C159" t="n">
-        <v>38.27790131944445</v>
+        <v>36.2064306</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>{9FED06B1-A2CE-4106-87D7-6B4CB6D55CCA}.jpg</t>
+          <t>{792B2B5E-02A8-4A3F-9477-F12B00E3600B}.jpg</t>
         </is>
       </c>
       <c r="B160" t="n">
-        <v>36.20873725000001</v>
+        <v>36.21945631944445</v>
       </c>
       <c r="C160" t="n">
-        <v>36.15536491666666</v>
+        <v>36.15724396388889</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>{792B2B5E-02A8-4A3F-9477-F12B00E3600B}.jpg</t>
+          <t>{413B2715-7F2A-4709-8956-064FEA2D5AF0}.jpg</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>36.21945631944445</v>
+        <v>37.76664772222222</v>
       </c>
       <c r="C161" t="n">
-        <v>36.15724396388889</v>
+        <v>38.27008745</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>{0C7D0626-0EAB-4625-8A01-26E1426B140D}.jpg</t>
+          <t>{DBE68764-1740-4D57-894C-0996AF790A55}.jpg</t>
         </is>
       </c>
       <c r="B162" t="n">
-        <v>36.20641963888889</v>
+        <v>36.5663675</v>
       </c>
       <c r="C162" t="n">
-        <v>36.15414376944445</v>
+        <v>36.15448655555556</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>{61202A8E-4B72-4066-ABDB-7E19D342398A}.jpg</t>
+          <t>{C0049CBE-AF03-4A7C-8A59-FB3067BA6CFA}.jpg</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>37.59148481944445</v>
+        <v>36.23541758333334</v>
       </c>
       <c r="C163" t="n">
-        <v>36.86722861</v>
+        <v>36.16584438888889</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>{DB70A36E-BB7F-47BE-9FB6-B95AB71EC53F}.jpg</t>
+          <t>{C651EBF2-F7EC-485A-9987-2E679E77CAB2}.jpg</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>36.21428611111111</v>
+        <v>37.58198327777778</v>
       </c>
       <c r="C164" t="n">
-        <v>36.13610555555555</v>
+        <v>36.97184808888889</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>{87FF0DDB-65FB-426B-A8CA-EC4B0426511A}.jpg</t>
+          <t>{4459907D-5404-4825-B34E-A427A45BCE6E}.jpg</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>36.23043216666667</v>
+        <v>37.76901559722222</v>
       </c>
       <c r="C165" t="n">
-        <v>36.14797288888889</v>
+        <v>38.28402379305555</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>{220782BB-3CED-4B7C-B1F9-5C55C0545FD2}.jpg</t>
+          <t>{D669053A-A9BA-4437-B80D-29D9F8A13CBC}.jpg</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>37.76109163888889</v>
+        <v>37.76528122222222</v>
       </c>
       <c r="C166" t="n">
-        <v>38.25722463888889</v>
+        <v>38.2711316</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>{292912A9-674E-4A41-89DD-7F0E0E550A84}.jpg</t>
+          <t>{625CBA71-1962-4E2D-B66B-F41750297B25}.jpg</t>
         </is>
       </c>
       <c r="B167" t="n">
-        <v>37.78029586111111</v>
+        <v>37.69185643055555</v>
       </c>
       <c r="C167" t="n">
-        <v>38.25637026944445</v>
+        <v>37.84913325</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>{C2B793BD-1F97-4430-BB56-FA30685BBA6F}.jpg</t>
+          <t>{41468389-970A-4898-B53E-D4BF30729BB9}.jpg</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>37.57351893055556</v>
+        <v>36.22845608333333</v>
       </c>
       <c r="C168" t="n">
-        <v>36.92560222222222</v>
+        <v>36.19931422222222</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>{B80ACF18-864C-4E62-BB4A-56820D4621C7}.jpg</t>
+          <t>{5F85BE1A-EE78-4FD7-8F28-C95BAD00EFB1}.jpg</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>36.19611305555555</v>
+        <v>37.57198225</v>
       </c>
       <c r="C169" t="n">
-        <v>36.15939951666667</v>
+        <v>36.93414867583333</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>{90440650-25E8-4A66-9322-D2531DE72CA6}.jpg</t>
+          <t>{D68EFBBB-8DFB-4F02-930D-AE9DDBDE858F}.jpg</t>
         </is>
       </c>
       <c r="B170" t="n">
-        <v>37.76381297222222</v>
+        <v>36.20416505555556</v>
       </c>
       <c r="C170" t="n">
-        <v>38.27171358888889</v>
+        <v>36.14976594444445</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>{869B730A-D1B9-4DFB-8841-1DD70CFEBD82}.jpg</t>
+          <t>{488CD3CA-D8CA-4237-9887-DAB6DB8ACBEC}.jpg</t>
         </is>
       </c>
       <c r="B171" t="n">
-        <v>36.21746742222222</v>
+        <v>37.57260736666667</v>
       </c>
       <c r="C171" t="n">
-        <v>36.14187011111111</v>
+        <v>36.93593906111111</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>{6269F227-5B6F-48A4-A5BA-4DA0F809ECA9}.jpg</t>
+          <t>{76385D9D-0839-4B82-ADF6-F3318D1EF23F}.jpg</t>
         </is>
       </c>
       <c r="B172" t="n">
-        <v>37.75710192777778</v>
+        <v>37.57472775</v>
       </c>
       <c r="C172" t="n">
-        <v>38.25502502777778</v>
+        <v>36.94820544444444</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>{E31AE50A-1982-4A70-B59B-424B598D1A40}.jpg</t>
+          <t>{4AD3B275-A164-4918-9993-06F17A29CB18}.jpg</t>
         </is>
       </c>
       <c r="B173" t="n">
-        <v>36.2173728</v>
+        <v>37.76141666666667</v>
       </c>
       <c r="C173" t="n">
-        <v>36.17171579999999</v>
+        <v>38.26574166666666</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>{C651EBF2-F7EC-485A-9987-2E679E77CAB2}.jpg</t>
+          <t>{9E525EE6-ED31-4103-86E1-0F89C53E89C2}.jpg</t>
         </is>
       </c>
       <c r="B174" t="n">
-        <v>37.58198327777778</v>
+        <v>37.76260077777778</v>
       </c>
       <c r="C174" t="n">
-        <v>36.97184808888889</v>
+        <v>38.29404586111111</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>{15FAFC51-6470-44F3-B24B-3EA00D097841}.jpg</t>
+          <t>{4CB47C59-F3E5-4CD3-BDEA-D1E647A12F29}.jpg</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>36.20613959166667</v>
+        <v>37.68756449999999</v>
       </c>
       <c r="C175" t="n">
-        <v>36.16995713333333</v>
+        <v>37.85580256388889</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>{09F10EDC-083A-4F26-BB6C-A9AE0CCD766B}.jpg</t>
+          <t>{B187F4FB-88CB-4548-A114-1FB9462487B1}.jpg</t>
         </is>
       </c>
       <c r="B176" t="n">
-        <v>37.57178513888889</v>
+        <v>37.58039016666667</v>
       </c>
       <c r="C176" t="n">
-        <v>36.93474944722222</v>
+        <v>36.9272646</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>{255CEE31-67B1-423D-8692-2A39F25CC46B}.jpg</t>
+          <t>{16C2E690-76CF-4A5E-B8A6-6E1AEAB58D1C}.jpg</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>36.22817019444444</v>
+        <v>37.77255085277778</v>
       </c>
       <c r="C177" t="n">
-        <v>36.1482965</v>
+        <v>38.26293702777778</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>{91801DA2-AABA-4497-8E2A-CFFDFE59AEFA}.jpg</t>
+          <t>{5E6BD6EA-F129-410F-9C93-13D4DE27771C}.jpg</t>
         </is>
       </c>
       <c r="B178" t="n">
-        <v>36.21507863888889</v>
+        <v>37.57328694444445</v>
       </c>
       <c r="C178" t="n">
-        <v>36.15871686111111</v>
+        <v>36.91925611944444</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>{140D61AC-0E19-4134-8EF7-656DB1323C44}.jpg</t>
+          <t>{0A76082E-A7E6-49E8-B505-DF818E9CFFC7}.jpg</t>
         </is>
       </c>
       <c r="B179" t="n">
-        <v>36.49513530555556</v>
+        <v>36.21239963888889</v>
       </c>
       <c r="C179" t="n">
-        <v>36.36784786944445</v>
+        <v>36.14170272222222</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>{187D9D93-53CC-4953-B80F-3A5107A7192D}.jpg</t>
+          <t>{8844779C-8F37-4EA8-9593-E82B97869B1B}.jpg</t>
         </is>
       </c>
       <c r="B180" t="n">
-        <v>36.25969455555555</v>
+        <v>36.25973622222222</v>
       </c>
       <c r="C180" t="n">
-        <v>36.20641123888889</v>
+        <v>36.20641127777778</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>{015EA546-5006-4ECD-A229-E87B39B802AA}.jpg</t>
+          <t>{67B4F126-D2C0-4B70-ACF0-4219ED828B48}.jpg</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>37.77459511111111</v>
+        <v>37.76154369444444</v>
       </c>
       <c r="C181" t="n">
-        <v>38.26554547222222</v>
+        <v>38.2412609</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>{DACF98B6-F238-496B-8AE1-9BD115939851}.jpg</t>
+          <t>{DE6237B2-43FB-407B-8D16-D0280AA530D0}.jpg</t>
         </is>
       </c>
       <c r="B182" t="n">
-        <v>36.21453055555556</v>
+        <v>36.23085997222223</v>
       </c>
       <c r="C182" t="n">
-        <v>36.14272777777778</v>
+        <v>36.19969302777778</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>{BD037D65-F49F-4928-9886-8C903F336B99}.jpg</t>
+          <t>{6269F227-5B6F-48A4-A5BA-4DA0F809ECA9}.jpg</t>
         </is>
       </c>
       <c r="B183" t="n">
-        <v>36.21493561111112</v>
+        <v>37.75710192777778</v>
       </c>
       <c r="C183" t="n">
-        <v>36.15828919444444</v>
+        <v>38.25502502777778</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>{C0049CBE-AF03-4A7C-8A59-FB3067BA6CFA}.jpg</t>
+          <t>{A0D18F36-EA14-4F20-8765-A379DCEAA9BB}.jpg</t>
         </is>
       </c>
       <c r="B184" t="n">
-        <v>36.23541758333334</v>
+        <v>36.23093380555556</v>
       </c>
       <c r="C184" t="n">
-        <v>36.16584438888889</v>
+        <v>36.20075208333333</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>{99BC0159-4837-439A-A0EF-9E5F01283C4C}.jpg</t>
+          <t>{D105F006-5C19-46D8-8C21-F1B4B050D4BF}.jpg</t>
         </is>
       </c>
       <c r="B185" t="n">
-        <v>36.19769127777777</v>
+        <v>36.22710269444445</v>
       </c>
       <c r="C185" t="n">
-        <v>36.16628202777778</v>
+        <v>36.151333</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>{EFDFFCBA-8E66-4285-861E-E0E108B3C0C6}.jpg</t>
+          <t>{FEE4E162-E515-44F6-B8C1-9A45932DF4E1}.jpg</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>37.76507219444444</v>
+        <v>37.69072601111111</v>
       </c>
       <c r="C186" t="n">
-        <v>38.2371099</v>
+        <v>37.84884450000001</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>{068E9554-8EFF-4FCE-9CDC-1101FD7FA241}.jpg</t>
+          <t>{6FFEFA7D-F17D-4627-B55D-3CD949C486D3}.jpg</t>
         </is>
       </c>
       <c r="B187" t="n">
-        <v>36.25975647222222</v>
+        <v>36.20325993055556</v>
       </c>
       <c r="C187" t="n">
-        <v>36.20639878888889</v>
+        <v>36.14778175</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>{EC37422A-5C73-47B5-9212-F7979C986E43}.jpg</t>
+          <t>{8677E52A-A4A6-47AE-B373-0A891D0BAE64}.jpg</t>
         </is>
       </c>
       <c r="B188" t="n">
-        <v>36.25974068055555</v>
+        <v>36.20174878888889</v>
       </c>
       <c r="C188" t="n">
-        <v>36.20637169444445</v>
+        <v>36.16428277777778</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>{81011EC3-C0CB-40B2-8ACB-34FACE9B1E9C}.jpg</t>
+          <t>{255CEE31-67B1-423D-8692-2A39F25CC46B}.jpg</t>
         </is>
       </c>
       <c r="B189" t="n">
-        <v>36.2263936</v>
+        <v>36.22817019444444</v>
       </c>
       <c r="C189" t="n">
-        <v>36.1510569</v>
+        <v>36.1482965</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>{51490BFF-82E7-4BEF-81D5-C1560BD38627}.jpg</t>
+          <t>{45EF9F99-7A3F-4A40-8402-B4B5621D6BFA}.jpg</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>37.57397816666667</v>
+        <v>37.74935630555556</v>
       </c>
       <c r="C190" t="n">
-        <v>36.93450889722222</v>
+        <v>38.25261056944444</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>{EE19E7FA-1771-4CA1-AB03-0A6A9EBF440E}.jpg</t>
+          <t>{81FBFA74-519D-447E-AB46-5F27487DAA06}.jpg</t>
         </is>
       </c>
       <c r="B191" t="n">
-        <v>36.22827563888889</v>
+        <v>37.75843316666667</v>
       </c>
       <c r="C191" t="n">
-        <v>36.15116346666667</v>
+        <v>38.27627540555555</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>{CBC9BA7D-56F2-4628-ADF1-235F4D89B84C}.jpg</t>
+          <t>{8CAAEAE1-FB3D-47EF-A12E-C5F7302E63EA}.jpg</t>
         </is>
       </c>
       <c r="B192" t="n">
-        <v>36.19663611111111</v>
+        <v>37.584649275</v>
       </c>
       <c r="C192" t="n">
-        <v>36.14903888888889</v>
+        <v>36.92915265277777</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>{4459907D-5404-4825-B34E-A427A45BCE6E}.jpg</t>
+          <t>{EE19E7FA-1771-4CA1-AB03-0A6A9EBF440E}.jpg</t>
         </is>
       </c>
       <c r="B193" t="n">
-        <v>37.76901559722222</v>
+        <v>36.22827563888889</v>
       </c>
       <c r="C193" t="n">
-        <v>38.28402379305555</v>
+        <v>36.15116346666667</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>{FEE4E162-E515-44F6-B8C1-9A45932DF4E1}.jpg</t>
+          <t>{420E37E1-0180-4B96-BD5E-434F1AEA915F}.jpg</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>37.69072601111111</v>
+        <v>37.77295201111111</v>
       </c>
       <c r="C194" t="n">
-        <v>37.84884450000001</v>
+        <v>38.26867796388889</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>{D301AEB0-492E-41E4-8D0C-009DEF9F0382}.jpg</t>
+          <t>{2A00B94E-8B01-4342-8E9E-6E3DEFAD2B09}.jpg</t>
         </is>
       </c>
       <c r="B195" t="n">
-        <v>37.57303544444445</v>
+        <v>37.75638319444445</v>
       </c>
       <c r="C195" t="n">
-        <v>36.93914701111111</v>
+        <v>38.2355974</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>{09B0A8BE-FC31-4BCD-9286-E6C3D6D4E400}.jpg</t>
+          <t>{F3A4956D-EDF2-468D-9FC4-F0169FED8F23}.jpg</t>
         </is>
       </c>
       <c r="B196" t="n">
-        <v>36.23008572222222</v>
+        <v>36.22723630555556</v>
       </c>
       <c r="C196" t="n">
-        <v>36.14873766666667</v>
+        <v>36.15126830555555</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>{A257A9FE-77C2-45EC-891E-9DC249A30005}.jpg</t>
+          <t>{C2B793BD-1F97-4430-BB56-FA30685BBA6F}.jpg</t>
         </is>
       </c>
       <c r="B197" t="n">
-        <v>37.57474166666667</v>
+        <v>37.57351893055556</v>
       </c>
       <c r="C197" t="n">
-        <v>36.93337166666667</v>
+        <v>36.92560222222222</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>{07AD392A-3C05-451D-836E-FED8051022F9}.jpg</t>
+          <t>{8323814C-3708-4EAB-B5B7-B6B0B2B9CB96}.jpg</t>
         </is>
       </c>
       <c r="B198" t="n">
-        <v>36.20226519166667</v>
+        <v>37.73547438333333</v>
       </c>
       <c r="C198" t="n">
-        <v>36.1641085</v>
+        <v>38.223239</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>{F1A12DB3-DF1C-4A07-939F-CE4C1E3E9F1F}.jpg</t>
+          <t>{C4EFA374-6F6C-45D4-B48F-82A60766854C}.jpg</t>
         </is>
       </c>
       <c r="B199" t="n">
-        <v>36.23472901666667</v>
+        <v>36.23690765833334</v>
       </c>
       <c r="C199" t="n">
-        <v>36.17125478611111</v>
+        <v>36.16569116666667</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>{0F20EE24-A6F5-434A-A8BC-A69A2233D152}.jpg</t>
+          <t>{93CA0A7E-EF3F-43AC-BE9B-5C7EE7DBC5E7}.jpg</t>
         </is>
       </c>
       <c r="B200" t="n">
-        <v>36.20747659166667</v>
+        <v>36.49920605555555</v>
       </c>
       <c r="C200" t="n">
-        <v>36.15842320555556</v>
+        <v>36.34610094444444</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>{4DA0D867-38B2-4389-9925-1ACE3FBCF202}.jpg</t>
+          <t>{EE051ED5-8815-4C5A-9044-1C37D8094737}.jpg</t>
         </is>
       </c>
       <c r="B201" t="n">
-        <v>36.20626212777778</v>
+        <v>36.19660688888889</v>
       </c>
       <c r="C201" t="n">
-        <v>36.15387052777778</v>
+        <v>36.14767</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>{CA3CF42C-1BAC-4300-8942-CF049F944ABD}.jpg</t>
+          <t>{0C7D0626-0EAB-4625-8A01-26E1426B140D}.jpg</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>36.21773038888889</v>
+        <v>36.20641963888889</v>
       </c>
       <c r="C202" t="n">
-        <v>36.15750787222222</v>
+        <v>36.15414376944445</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>{A0E9FC65-1668-4425-95A2-92754032167E}.jpg</t>
+          <t>{87FF0DDB-65FB-426B-A8CA-EC4B0426511A}.jpg</t>
         </is>
       </c>
       <c r="B203" t="n">
-        <v>37.76592977777778</v>
+        <v>36.23043216666667</v>
       </c>
       <c r="C203" t="n">
-        <v>38.26638852777778</v>
+        <v>36.14797288888889</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>{FF3046E1-7C71-44D6-BDBF-21E92799D7E1}.jpg</t>
+          <t>{C0321E11-988C-4759-BD4F-48BE594C83C0}.jpg</t>
         </is>
       </c>
       <c r="B204" t="n">
-        <v>36.22242430555556</v>
+        <v>37.75964598888889</v>
       </c>
       <c r="C204" t="n">
-        <v>36.1543973</v>
+        <v>38.25997297222222</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>{8CAAEAE1-FB3D-47EF-A12E-C5F7302E63EA}.jpg</t>
+          <t>{ED3AF46A-8F29-4E18-91D4-CF69715C7122}.jpg</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>37.584649275</v>
+        <v>36.25974952777778</v>
       </c>
       <c r="C205" t="n">
-        <v>36.92915265277777</v>
+        <v>36.20640106944445</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>{308DFE10-3912-43E5-B668-A60098830163}.jpg</t>
+          <t>{5E62109E-E85D-4B02-B728-5C9924E46640}.jpg</t>
         </is>
       </c>
       <c r="B206" t="n">
-        <v>37.75711963055556</v>
+        <v>36.25972930555555</v>
       </c>
       <c r="C206" t="n">
-        <v>38.25622673333334</v>
+        <v>36.20641543055556</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>{9AEB2EA6-67A4-402D-86DF-66F3AD34A946}.jpg</t>
+          <t>{E316E926-E8EE-4EA4-B951-0736886C9B20}.jpg</t>
         </is>
       </c>
       <c r="B207" t="n">
-        <v>37.76503930555555</v>
+        <v>37.55946666666667</v>
       </c>
       <c r="C207" t="n">
-        <v>38.2371118</v>
+        <v>36.9209</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>{8ABA5D32-68F5-4B8C-8E2B-33335818C3A6}.jpg</t>
+          <t>{45A41380-3CD2-45F5-8ADF-F6AC5FA95246}.jpg</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>36.2157633888889</v>
+        <v>36.20962196111111</v>
       </c>
       <c r="C208" t="n">
-        <v>36.1574949</v>
+        <v>36.16005752777777</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>{F6CA6BB0-293B-43A4-9C62-53F015D6A646}.jpg</t>
+          <t>{796E0D03-8A48-4073-BDEC-E2BF1FB9CD00}.jpg</t>
         </is>
       </c>
       <c r="B209" t="n">
-        <v>37.58136727777778</v>
+        <v>37.77280960277778</v>
       </c>
       <c r="C209" t="n">
-        <v>36.96623416666667</v>
+        <v>38.26867109166667</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>{4CB47C59-F3E5-4CD3-BDEA-D1E647A12F29}.jpg</t>
+          <t>{C2EEF875-FCC6-4CF2-A186-334FFC456E56}.jpg</t>
         </is>
       </c>
       <c r="B210" t="n">
-        <v>37.68756449999999</v>
+        <v>36.25975455555555</v>
       </c>
       <c r="C210" t="n">
-        <v>37.85580256388889</v>
+        <v>36.20638661944444</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>{5A930121-C734-45E3-9853-12C2E4F0721C}.jpg</t>
+          <t>{F1A12DB3-DF1C-4A07-939F-CE4C1E3E9F1F}.jpg</t>
         </is>
       </c>
       <c r="B211" t="n">
-        <v>36.22788936111111</v>
+        <v>36.23472901666667</v>
       </c>
       <c r="C211" t="n">
-        <v>36.14941116666667</v>
+        <v>36.17125478611111</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>{C24A026F-473B-420A-9021-B8D1E0D87556}.jpg</t>
+          <t>{C3283350-EC30-4BE6-B17C-BAC34AAE6747}.jpg</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>36.21751410388889</v>
+        <v>37.57517511111111</v>
       </c>
       <c r="C212" t="n">
-        <v>36.15671741666667</v>
+        <v>36.93200433333333</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>{12D329B8-7451-468E-B226-530A2D215515}.jpg</t>
+          <t>{6C7C5BA8-7A25-4537-85ED-46A171F702C6}.jpg</t>
         </is>
       </c>
       <c r="B213" t="n">
-        <v>36.25971043055556</v>
+        <v>36.19630394444444</v>
       </c>
       <c r="C213" t="n">
-        <v>36.2064306</v>
+        <v>36.15433265</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>{45EF9F99-7A3F-4A40-8402-B4B5621D6BFA}.jpg</t>
+          <t>{0F2ADD6B-076F-4A45-B91D-7C63B32CB26F}.jpg</t>
         </is>
       </c>
       <c r="B214" t="n">
-        <v>37.74935630555556</v>
+        <v>36.20645642777778</v>
       </c>
       <c r="C214" t="n">
-        <v>38.25261056944444</v>
+        <v>36.15686209722222</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>{B5D8A6DA-7663-4EAB-91A1-45AF7DEB0A9B}.jpg</t>
+          <t>{DA075791-5464-410E-AA19-726B5B154045}.jpg</t>
         </is>
       </c>
       <c r="B215" t="n">
-        <v>36.19685419444444</v>
+        <v>36.20225089722223</v>
       </c>
       <c r="C215" t="n">
-        <v>36.15055765833333</v>
+        <v>36.14826561111111</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>{4E66CC9B-DCB4-404C-B9E3-23DF6CE285C3}.jpg</t>
+          <t>{C24A026F-473B-420A-9021-B8D1E0D87556}.jpg</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>37.57212277777778</v>
+        <v>36.21751410388889</v>
       </c>
       <c r="C216" t="n">
-        <v>36.93805176944444</v>
+        <v>36.15671741666667</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>{616A9B44-8575-4C2E-8CDB-188AAB7FB426}.jpg</t>
+          <t>{CD574077-0E65-4263-8E08-DF099D9B31B4}.jpg</t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>37.74692608333334</v>
+        <v>36.20633603611111</v>
       </c>
       <c r="C217" t="n">
-        <v>38.24972905555556</v>
+        <v>36.15694974166666</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>{D105F006-5C19-46D8-8C21-F1B4B050D4BF}.jpg</t>
+          <t>{C40C3F47-F5F4-4194-B2A9-09D274C6650A}.jpg</t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>36.22710269444445</v>
+        <v>37.0627124</v>
       </c>
       <c r="C218" t="n">
-        <v>36.151333</v>
+        <v>36.23670659972223</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>{DD273D01-328C-4813-8E3F-3A16DB0DCD7C}.jpg</t>
+          <t>{26BCBA63-E13F-4E7B-A019-BE7A4C63A053}.jpg</t>
         </is>
       </c>
       <c r="B219" t="n">
-        <v>37.76882104722222</v>
+        <v>37.570865</v>
       </c>
       <c r="C219" t="n">
-        <v>38.26127321111111</v>
+        <v>36.91841333333333</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>{8C24F76B-9E22-472B-AFF8-3D2824820793}.jpg</t>
+          <t>{C165CBE8-C191-4C8A-AD79-ACB5DC61936C}.jpg</t>
         </is>
       </c>
       <c r="B220" t="n">
-        <v>36.21900767222223</v>
+        <v>37.58274658333334</v>
       </c>
       <c r="C220" t="n">
-        <v>36.15748983333333</v>
+        <v>36.88289466666667</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>{B1D62FB5-6F0F-408A-BBF3-BF2F64BA5012}.jpg</t>
+          <t>{9E270B5D-22BB-4F5B-A895-962198E7C09A}.jpg</t>
         </is>
       </c>
       <c r="B221" t="n">
-        <v>37.76829</v>
+        <v>37.76945508333333</v>
       </c>
       <c r="C221" t="n">
-        <v>38.26105833333333</v>
+        <v>38.26309669444444</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>{50930D18-9C78-436D-BD9D-6AE5EC2C74FC}.jpg</t>
+          <t>{440E99B0-8701-492A-BBC4-5DB76137C7CA}.jpg</t>
         </is>
       </c>
       <c r="B222" t="n">
-        <v>36.20350825000001</v>
+        <v>36.56693796694445</v>
       </c>
       <c r="C222" t="n">
-        <v>36.15870213888888</v>
+        <v>36.15080136305556</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>{67B4F126-D2C0-4B70-ACF0-4219ED828B48}.jpg</t>
+          <t>{BE32E2E9-8598-457A-AC40-94DE5C1BFC47}.jpg</t>
         </is>
       </c>
       <c r="B223" t="n">
-        <v>37.76154369444444</v>
+        <v>37.76414308333333</v>
       </c>
       <c r="C223" t="n">
-        <v>38.2412609</v>
+        <v>38.27738761111111</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>{420E37E1-0180-4B96-BD5E-434F1AEA915F}.jpg</t>
+          <t>{90440650-25E8-4A66-9322-D2531DE72CA6}.jpg</t>
         </is>
       </c>
       <c r="B224" t="n">
-        <v>37.77295201111111</v>
+        <v>37.76381297222222</v>
       </c>
       <c r="C224" t="n">
-        <v>38.26867796388889</v>
+        <v>38.27171358888889</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>{83A27DD6-A1E4-4A52-B89B-33EA3E12EAE2}.jpg</t>
+          <t>{61202A8E-4B72-4066-ABDB-7E19D342398A}.jpg</t>
         </is>
       </c>
       <c r="B225" t="n">
-        <v>36.21117308333334</v>
+        <v>37.59148481944445</v>
       </c>
       <c r="C225" t="n">
-        <v>36.14328265555555</v>
+        <v>36.86722861</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>{6DE016A3-15FD-4DB6-B0FE-40295FFE37D1}.jpg</t>
+          <t>{A289263E-4C12-4525-ADAB-E912A19D1D58}.jpg</t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>36.20635880555556</v>
+        <v>37.56425166666666</v>
       </c>
       <c r="C226" t="n">
-        <v>36.15690767222222</v>
+        <v>36.921615</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>{1E214BAA-AEE7-41AE-90B3-8E1C6D0FBB29}.jpg</t>
+          <t>{EE373BCB-3DB3-49EB-8390-A62561B0A358}.jpg</t>
         </is>
       </c>
       <c r="B227" t="n">
-        <v>36.25973786111111</v>
+        <v>37.55979833333333</v>
       </c>
       <c r="C227" t="n">
-        <v>36.20640465</v>
+        <v>36.91985833333333</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>{F35C84A1-4459-4B1B-B70E-55531F735CD6}.jpg</t>
+          <t>{D17BB85F-B73B-49CD-855C-5136B6F634A2}.jpg</t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>37.48986666666666</v>
+        <v>36.21758978888889</v>
       </c>
       <c r="C228" t="n">
-        <v>37.07037833333334</v>
+        <v>36.157137925</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>{80EAEDD9-1807-45E1-88AD-55006C712D03}.jpg</t>
+          <t>{F35C84A1-4459-4B1B-B70E-55531F735CD6}.jpg</t>
         </is>
       </c>
       <c r="B229" t="n">
-        <v>37.76325691666667</v>
+        <v>37.48986666666666</v>
       </c>
       <c r="C229" t="n">
-        <v>38.28148530555556</v>
+        <v>37.07037833333334</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>{1D8F887A-9D75-448A-87A8-33AEBC6ABFB4}.jpg</t>
+          <t>{91801DA2-AABA-4497-8E2A-CFFDFE59AEFA}.jpg</t>
         </is>
       </c>
       <c r="B230" t="n">
-        <v>37.5718793888889</v>
+        <v>36.21507863888889</v>
       </c>
       <c r="C230" t="n">
-        <v>36.92210701944444</v>
+        <v>36.15871686111111</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>{5E62109E-E85D-4B02-B728-5C9924E46640}.jpg</t>
+          <t>{73999AD7-A08F-455C-8B27-B675417BE7AC}.jpg</t>
         </is>
       </c>
       <c r="B231" t="n">
-        <v>36.25972930555555</v>
+        <v>37.765515</v>
       </c>
       <c r="C231" t="n">
-        <v>36.20641543055556</v>
+        <v>38.26564933333334</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>{7BC03BE0-EBB4-4F80-850D-B1D3F41C7602}.jpg</t>
+          <t>{E851A14E-6C4F-4FA0-95FF-18957BE4EFE1}.jpg</t>
         </is>
       </c>
       <c r="B232" t="n">
-        <v>36.22872155555556</v>
+        <v>37.76634361111111</v>
       </c>
       <c r="C232" t="n">
-        <v>36.15095917777778</v>
+        <v>38.27160925</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>{73999AD7-A08F-455C-8B27-B675417BE7AC}.jpg</t>
+          <t>{308DFE10-3912-43E5-B668-A60098830163}.jpg</t>
         </is>
       </c>
       <c r="B233" t="n">
-        <v>37.765515</v>
+        <v>37.75711963055556</v>
       </c>
       <c r="C233" t="n">
-        <v>38.26564933333334</v>
+        <v>38.25622673333334</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>{13B0F93E-52A9-4884-AFC5-661AC641A905}.jpg</t>
+          <t>{992B9E79-CF5B-44F7-B2C3-9F0D28A1A12E}.jpg</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>37.75872943055555</v>
+        <v>36.25974716666666</v>
       </c>
       <c r="C234" t="n">
-        <v>38.26542552777778</v>
+        <v>36.20638947222223</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>{B187F4FB-88CB-4548-A114-1FB9462487B1}.jpg</t>
+          <t>{9BE883AD-4F74-4CBA-B93B-0FAC129B556A}.jpg</t>
         </is>
       </c>
       <c r="B235" t="n">
-        <v>37.58039016666667</v>
+        <v>37.77066572222222</v>
       </c>
       <c r="C235" t="n">
-        <v>36.9272646</v>
+        <v>38.26634486111111</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>{A9078FAA-C0C7-4EB0-87EB-2D936A70B2CA}.jpg</t>
+          <t>{66EE713E-4CE2-4DF5-97D9-196311459D20}.jpg</t>
         </is>
       </c>
       <c r="B236" t="n">
-        <v>37.68828020555555</v>
+        <v>37.761505</v>
       </c>
       <c r="C236" t="n">
-        <v>37.85578821388889</v>
+        <v>38.26583666666667</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>{F3A4956D-EDF2-468D-9FC4-F0169FED8F23}.jpg</t>
+          <t>{3F02D8E9-773E-47CD-8946-841459249D09}.jpg</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>36.22723630555556</v>
+        <v>36.20548883333333</v>
       </c>
       <c r="C237" t="n">
-        <v>36.15126830555555</v>
+        <v>36.15434047777778</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>{8C45868F-979A-432F-8C42-4B0DEFA80225}.jpg</t>
+          <t>{99BC0159-4837-439A-A0EF-9E5F01283C4C}.jpg</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>36.20622158333334</v>
+        <v>36.19769127777777</v>
       </c>
       <c r="C238" t="n">
-        <v>36.17344077777778</v>
+        <v>36.16628202777778</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>{A0678E82-032A-4D3A-B176-A9FA1FE066D9}.jpg</t>
+          <t>{CCE1D552-EEA7-4EB0-B337-B91E6357B702}.jpg</t>
         </is>
       </c>
       <c r="B239" t="n">
-        <v>37.76613088888889</v>
+        <v>36.25973426111111</v>
       </c>
       <c r="C239" t="n">
-        <v>38.266975575</v>
+        <v>36.20640416111112</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>{F0EF1E9D-1E57-47FC-8439-244452934513}.jpg</t>
+          <t>{DB70A36E-BB7F-47BE-9FB6-B95AB71EC53F}.jpg</t>
         </is>
       </c>
       <c r="B240" t="n">
-        <v>36.19645522222222</v>
+        <v>36.21428611111111</v>
       </c>
       <c r="C240" t="n">
-        <v>36.16005752777777</v>
+        <v>36.13610555555555</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>{0450CBDA-5560-41B1-9C27-00C1B01BC741}.jpg</t>
+          <t>{50930D18-9C78-436D-BD9D-6AE5EC2C74FC}.jpg</t>
         </is>
       </c>
       <c r="B241" t="n">
-        <v>37.76594458333334</v>
+        <v>36.20350825000001</v>
       </c>
       <c r="C241" t="n">
-        <v>38.26616363888889</v>
+        <v>36.15870213888888</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>{907FEA05-9978-418E-923A-006E5907B677}.jpg</t>
+          <t>{82117B6A-CB2C-456F-9DAA-DBDA8C206503}.jpg</t>
         </is>
       </c>
       <c r="B242" t="n">
-        <v>37.57328095277778</v>
+        <v>36.19532788888888</v>
       </c>
       <c r="C242" t="n">
-        <v>36.91966454444444</v>
+        <v>36.15280598888889</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>{561F2B1A-FA0F-4657-B868-1510ADC53059}.jpg</t>
+          <t>{E1038CCD-0C6D-4E1E-A89F-4AF5F7B06564}.jpg</t>
         </is>
       </c>
       <c r="B243" t="n">
-        <v>36.21383997222222</v>
+        <v>37.76154788888889</v>
       </c>
       <c r="C243" t="n">
-        <v>36.15835197222222</v>
+        <v>38.24128419444445</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>{1FA33693-AB21-4438-8309-D5B670E14256}.jpg</t>
+          <t>{EFDFFCBA-8E66-4285-861E-E0E108B3C0C6}.jpg</t>
         </is>
       </c>
       <c r="B244" t="n">
-        <v>36.20757777777778</v>
+        <v>37.76507219444444</v>
       </c>
       <c r="C244" t="n">
-        <v>36.15067222222222</v>
+        <v>38.2371099</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>{08093F3E-19B2-48AE-9016-EE21BA251891}.jpg</t>
+          <t>{E5D2916C-514A-4A1A-890F-E4A6DEF0F8D1}.jpg</t>
         </is>
       </c>
       <c r="B245" t="n">
-        <v>36.21840556666667</v>
+        <v>37.76167088888889</v>
       </c>
       <c r="C245" t="n">
-        <v>36.14167557222222</v>
+        <v>38.26634933333333</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>{FF3C2B33-5A26-4D71-B0E1-ADEA5B8815DB}.jpg</t>
+          <t>{787702D3-C98A-4B4F-809D-23B8358B4666}.jpg</t>
         </is>
       </c>
       <c r="B246" t="n">
-        <v>36.23030038888889</v>
+        <v>37.76055713888889</v>
       </c>
       <c r="C246" t="n">
-        <v>36.16433786111111</v>
+        <v>38.24986230555556</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>{5E830776-FCE1-480F-9B52-9B76D84C0BCD}.jpg</t>
+          <t>{B5D8A6DA-7663-4EAB-91A1-45AF7DEB0A9B}.jpg</t>
         </is>
       </c>
       <c r="B247" t="n">
-        <v>36.2597279</v>
+        <v>36.19685419444444</v>
       </c>
       <c r="C247" t="n">
-        <v>36.20637535</v>
+        <v>36.15055765833333</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>{EB274B9F-248D-4EB9-B173-53CC6BC5035C}.jpg</t>
+          <t>{55E6D05F-34D4-4933-8676-3C22C672929E}.jpg</t>
         </is>
       </c>
       <c r="B248" t="n">
-        <v>37.77169581388889</v>
+        <v>37.76337769444444</v>
       </c>
       <c r="C248" t="n">
-        <v>38.26375855555555</v>
+        <v>38.24220380555555</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>{F180F6DF-60C9-483C-A4E8-679B207DB9A7}.jpg</t>
+          <t>{56505110-B3B3-4565-A085-6AB8FF6D1465}.jpg</t>
         </is>
       </c>
       <c r="B249" t="n">
-        <v>36.19751488888888</v>
+        <v>36.21604819444445</v>
       </c>
       <c r="C249" t="n">
-        <v>36.16060378888888</v>
+        <v>36.15878076666667</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>{EC63F45D-EE35-4AB7-8652-339A19EC0235}.jpg</t>
+          <t>{4DA0D867-38B2-4389-9925-1ACE3FBCF202}.jpg</t>
         </is>
       </c>
       <c r="B250" t="n">
-        <v>37.752323</v>
+        <v>36.20626212777778</v>
       </c>
       <c r="C250" t="n">
-        <v>38.24599119444444</v>
+        <v>36.15387052777778</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>{451DBC30-C4F6-4961-8B2D-D223D5B3D20C}.jpg</t>
+          <t>{6944C862-D2C6-40CB-AC68-905DD2D3C36B}.jpg</t>
         </is>
       </c>
       <c r="B251" t="n">
-        <v>36.19433488888888</v>
+        <v>37.41076</v>
       </c>
       <c r="C251" t="n">
-        <v>36.15159435</v>
+        <v>36.88839</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>{C67DFB9D-E530-4330-A776-E060E638A9DC}.jpg</t>
+          <t>{09BA246A-63EB-4C38-9ED9-CB5A905081B8}.jpg</t>
         </is>
       </c>
       <c r="B252" t="n">
-        <v>37.76940508333333</v>
+        <v>37.78045788888889</v>
       </c>
       <c r="C252" t="n">
-        <v>38.25847466666666</v>
+        <v>38.25664012777778</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>{81FBFA74-519D-447E-AB46-5F27487DAA06}.jpg</t>
+          <t>{81941BBB-5130-47D0-8A5E-F39E9BC214A8}.jpg</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>37.75843316666667</v>
+        <v>36.21663263888889</v>
       </c>
       <c r="C253" t="n">
-        <v>38.27627540555555</v>
+        <v>36.16098418333333</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>{6944C862-D2C6-40CB-AC68-905DD2D3C36B}.jpg</t>
+          <t>{BBD96776-C4A8-40A8-AEE2-95C783C30AD6}.jpg</t>
         </is>
       </c>
       <c r="B254" t="n">
-        <v>37.41076</v>
+        <v>36.21687546861111</v>
       </c>
       <c r="C254" t="n">
-        <v>36.88839</v>
+        <v>36.16106102777778</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>{488CD3CA-D8CA-4237-9887-DAB6DB8ACBEC}.jpg</t>
+          <t>{F8E6D8C1-7DC7-40D2-9BE2-A7D5F653E380}.jpg</t>
         </is>
       </c>
       <c r="B255" t="n">
-        <v>37.57260736666667</v>
+        <v>36.25972861111111</v>
       </c>
       <c r="C255" t="n">
-        <v>36.93593906111111</v>
+        <v>36.20639278888889</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>{66EE713E-4CE2-4DF5-97D9-196311459D20}.jpg</t>
+          <t>{60692F62-3CBD-4B7A-B30B-66C3CA72BD9F}.jpg</t>
         </is>
       </c>
       <c r="B256" t="n">
-        <v>37.761505</v>
+        <v>36.218100825</v>
       </c>
       <c r="C256" t="n">
-        <v>38.26583666666667</v>
+        <v>36.15625135555555</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>{E6F5A316-85F0-4566-978A-18CCD49F1DC3}.jpg</t>
+          <t>{8CBE25CB-016C-4B12-AFA7-AAEFCAE027E6}.jpg</t>
         </is>
       </c>
       <c r="B257" t="n">
-        <v>37.76822578055555</v>
+        <v>36.21739308166667</v>
       </c>
       <c r="C257" t="n">
-        <v>38.26071347222222</v>
+        <v>36.15651826388888</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>{15FBDDE2-574A-4703-BC41-B676FE4C1B36}.jpg</t>
+          <t>{616A9B44-8575-4C2E-8CDB-188AAB7FB426}.jpg</t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>37.5872535</v>
+        <v>37.74692608333334</v>
       </c>
       <c r="C258" t="n">
-        <v>36.94399566666667</v>
+        <v>38.24972905555556</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>{D17BB85F-B73B-49CD-855C-5136B6F634A2}.jpg</t>
+          <t>{DD273D01-328C-4813-8E3F-3A16DB0DCD7C}.jpg</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>36.21758978888889</v>
+        <v>37.76882104722222</v>
       </c>
       <c r="C259" t="n">
-        <v>36.157137925</v>
+        <v>38.26127321111111</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>{C4EFA374-6F6C-45D4-B48F-82A60766854C}.jpg</t>
+          <t>{B91E6057-C51E-4712-AE63-EA2D8CC1E02B}.jpg</t>
         </is>
       </c>
       <c r="B260" t="n">
-        <v>36.23690765833334</v>
+        <v>36.23151038888889</v>
       </c>
       <c r="C260" t="n">
-        <v>36.16569116666667</v>
+        <v>36.16660011111111</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>{FE961C6B-6B7A-4D76-9A8F-AE33749201C2}.jpg</t>
+          <t>{0D8DCDB2-5D00-4625-88FD-66954466246B}.jpg</t>
         </is>
       </c>
       <c r="B261" t="n">
-        <v>36.22756836111111</v>
+        <v>36.22944644444445</v>
       </c>
       <c r="C261" t="n">
-        <v>36.15120042777777</v>
+        <v>36.16881010555555</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>{83552A61-02F9-40ED-AE40-C2CC166BE169}.jpg</t>
+          <t>{B20D4951-A7BD-4036-972A-9EBB2AEAFF99}.jpg</t>
         </is>
       </c>
       <c r="B262" t="n">
-        <v>36.19743413888889</v>
+        <v>36.20639013888889</v>
       </c>
       <c r="C262" t="n">
-        <v>36.15210824722222</v>
+        <v>36.15693141666667</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>{6806A4A9-CD94-4360-B74D-83BF39DAF537}.jpg</t>
+          <t>{5A930121-C734-45E3-9853-12C2E4F0721C}.jpg</t>
         </is>
       </c>
       <c r="B263" t="n">
-        <v>36.21795554444444</v>
+        <v>36.22788936111111</v>
       </c>
       <c r="C263" t="n">
-        <v>36.15632415555555</v>
+        <v>36.14941116666667</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>{DDA542AC-C3F9-4589-8893-91160E066A98}.jpg</t>
+          <t>{2C076564-83C0-41A5-AA77-05B8090B1AED}.jpg</t>
         </is>
       </c>
       <c r="B264" t="n">
-        <v>36.20597419444444</v>
+        <v>37.74773097222222</v>
       </c>
       <c r="C264" t="n">
-        <v>36.16011886111111</v>
+        <v>38.24966688888889</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>{8844779C-8F37-4EA8-9593-E82B97869B1B}.jpg</t>
+          <t>{1FA33693-AB21-4438-8309-D5B670E14256}.jpg</t>
         </is>
       </c>
       <c r="B265" t="n">
-        <v>36.25973622222222</v>
+        <v>36.20757777777778</v>
       </c>
       <c r="C265" t="n">
-        <v>36.20641127777778</v>
+        <v>36.15067222222222</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>{7E845995-5476-43EA-A08F-0AEB26D8E996}.jpg</t>
+          <t>{E956CAA0-2EDF-4A8F-8FCA-A1EC7F9F80EA}.jpg</t>
         </is>
       </c>
       <c r="B266" t="n">
-        <v>36.20154177222223</v>
+        <v>37.57699175</v>
       </c>
       <c r="C266" t="n">
-        <v>36.16488152777777</v>
+        <v>36.91670757722222</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>{52F3CCD8-4205-48B5-BDD3-700E4C072A59}.jpg</t>
+          <t>{3D4584B3-BE53-46C0-BB59-D8A9D355B08A}.jpg</t>
         </is>
       </c>
       <c r="B267" t="n">
-        <v>37.76945910555555</v>
+        <v>36.23589883333334</v>
       </c>
       <c r="C267" t="n">
-        <v>38.26838568888889</v>
+        <v>36.16497836111111</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>{ED3AF46A-8F29-4E18-91D4-CF69715C7122}.jpg</t>
+          <t>{396528FE-159B-4406-AF75-9EE1279E7ED9}.jpg</t>
         </is>
       </c>
       <c r="B268" t="n">
-        <v>36.25974952777778</v>
+        <v>37.76869134444444</v>
       </c>
       <c r="C268" t="n">
-        <v>36.20640106944445</v>
+        <v>38.26108356944444</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>{625CBA71-1962-4E2D-B66B-F41750297B25}.jpg</t>
+          <t>{ECF3A29B-3481-4627-89C9-1595B4880DD2}.jpg</t>
         </is>
       </c>
       <c r="B269" t="n">
-        <v>37.69185643055555</v>
+        <v>37.7531797</v>
       </c>
       <c r="C269" t="n">
-        <v>37.84913325</v>
+        <v>38.24628711111112</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>{F13B5AD2-FC07-4102-BD96-3484E1E0DEB4}.jpg</t>
+          <t>{83552A61-02F9-40ED-AE40-C2CC166BE169}.jpg</t>
         </is>
       </c>
       <c r="B270" t="n">
-        <v>37.76299483333333</v>
+        <v>36.19743413888889</v>
       </c>
       <c r="C270" t="n">
-        <v>38.29020973055555</v>
+        <v>36.15210824722222</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>{B20D4951-A7BD-4036-972A-9EBB2AEAFF99}.jpg</t>
+          <t>{89A572CB-D830-4737-BB40-A0597F77CB72}.jpg</t>
         </is>
       </c>
       <c r="B271" t="n">
-        <v>36.20639013888889</v>
+        <v>37.58176808333334</v>
       </c>
       <c r="C271" t="n">
-        <v>36.15693141666667</v>
+        <v>36.96571811111112</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>{9BE883AD-4F74-4CBA-B93B-0FAC129B556A}.jpg</t>
+          <t>{54C29DE1-D371-4A72-801B-97570E29D5BC}.jpg</t>
         </is>
       </c>
       <c r="B272" t="n">
-        <v>37.77066572222222</v>
+        <v>37.76448388888889</v>
       </c>
       <c r="C272" t="n">
-        <v>38.26634486111111</v>
+        <v>38.2355288</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>{0D8DCDB2-5D00-4625-88FD-66954466246B}.jpg</t>
+          <t>{A7FA99B1-A07B-42D6-AD97-53EBB6227CBD}.jpg</t>
         </is>
       </c>
       <c r="B273" t="n">
-        <v>36.22944644444445</v>
+        <v>37.68800143888888</v>
       </c>
       <c r="C273" t="n">
-        <v>36.16881010555555</v>
+        <v>37.85607461944445</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>{454A120C-20F7-499F-9CA3-70C771A7FD3A}.jpg</t>
+          <t>{C67DFB9D-E530-4330-A776-E060E638A9DC}.jpg</t>
         </is>
       </c>
       <c r="B274" t="n">
-        <v>36.20568175</v>
+        <v>37.76940508333333</v>
       </c>
       <c r="C274" t="n">
-        <v>36.15529327777778</v>
+        <v>38.25847466666666</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>{21254F46-EE21-4441-984B-01841C143E16}.jpg</t>
+          <t>{1243072D-C509-4AD1-BE81-83F18A77CB71}.jpg</t>
         </is>
       </c>
       <c r="B275" t="n">
-        <v>36.2037808</v>
+        <v>36.19771411111111</v>
       </c>
       <c r="C275" t="n">
-        <v>36.160363</v>
+        <v>36.1636545</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>{4DC84356-E1BD-4BAB-92BE-745F9604D49C}.jpg</t>
+          <t>{15FAFC51-6470-44F3-B24B-3EA00D097841}.jpg</t>
         </is>
       </c>
       <c r="B276" t="n">
-        <v>37.09941488888889</v>
+        <v>36.20613959166667</v>
       </c>
       <c r="C276" t="n">
-        <v>36.63670741111111</v>
+        <v>36.16995713333333</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>{796E0D03-8A48-4073-BDEC-E2BF1FB9CD00}.jpg</t>
+          <t>{C17DE65C-762E-41D9-A6FA-CCD9B77F5D62}.jpg</t>
         </is>
       </c>
       <c r="B277" t="n">
-        <v>37.77280960277778</v>
+        <v>37.76400797222222</v>
       </c>
       <c r="C277" t="n">
-        <v>38.26867109166667</v>
+        <v>38.27790131944445</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>{D669053A-A9BA-4437-B80D-29D9F8A13CBC}.jpg</t>
+          <t>{8C24F76B-9E22-472B-AFF8-3D2824820793}.jpg</t>
         </is>
       </c>
       <c r="B278" t="n">
-        <v>37.76528122222222</v>
+        <v>36.21900767222223</v>
       </c>
       <c r="C278" t="n">
-        <v>38.2711316</v>
+        <v>36.15748983333333</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>{50ABCC39-1DB7-4A13-944E-53EAB603ED2E}.jpg</t>
+          <t>{B2B3C2E9-5A4C-4889-BCC2-38A29B3300C8}.jpg</t>
         </is>
       </c>
       <c r="B279" t="n">
-        <v>36.21288877777778</v>
+        <v>36.19560213888889</v>
       </c>
       <c r="C279" t="n">
-        <v>36.14085708333333</v>
+        <v>36.15956888888888</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>{1FD1218E-ACF9-40D0-B4B4-106C37BD8878}.jpg</t>
+          <t>{FF3C2B33-5A26-4D71-B0E1-ADEA5B8815DB}.jpg</t>
         </is>
       </c>
       <c r="B280" t="n">
-        <v>37.57193877777778</v>
+        <v>36.23030038888889</v>
       </c>
       <c r="C280" t="n">
-        <v>36.91998378888889</v>
+        <v>36.16433786111111</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>{82C32338-B145-4825-8515-E49CDDE68032}.jpg</t>
+          <t>{DDA542AC-C3F9-4589-8893-91160E066A98}.jpg</t>
         </is>
       </c>
       <c r="B281" t="n">
-        <v>36.23181541666667</v>
+        <v>36.20597419444444</v>
       </c>
       <c r="C281" t="n">
-        <v>36.16548463888888</v>
+        <v>36.16011886111111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>